<commit_message>
Fix minor issues in excel tests.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
+++ b/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA034030-AED7-4F5C-B463-3410F44D59C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989D1F3F-D783-4A3B-BEEB-8FB51FCDD782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="-19455" windowWidth="28830" windowHeight="16335" activeTab="1" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="J13" s="33" cm="1">
         <f t="array" ref="J13">_xll.qlYieldTermStructureZeroRate($C$14,I13,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9561815272934002E-2</v>
+        <v>1.9561814398052216E-2</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="J14" s="33" cm="1">
         <f t="array" ref="J14">_xll.qlYieldTermStructureZeroRate($C$14,I14,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9508413641961174E-2</v>
+        <v>1.9508413197557743E-2</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="J15" s="33" cm="1">
         <f t="array" ref="J15">_xll.qlYieldTermStructureZeroRate($C$14,I15,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.942332976750076E-2</v>
+        <v>1.9423329540682495E-2</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="J16" s="33" cm="1">
         <f t="array" ref="J16">_xll.qlYieldTermStructureZeroRate($C$14,I16,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9516571239144988E-2</v>
+        <v>1.9707419970420838E-2</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="J17" s="33" cm="1">
         <f t="array" ref="J17">_xll.qlYieldTermStructureZeroRate($C$14,I17,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9929171494420136E-2</v>
+        <v>2.0304501541429942E-2</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J18" s="33" cm="1">
         <f t="array" ref="J18">_xll.qlYieldTermStructureZeroRate($C$14,I18,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0430384737421706E-2</v>
+        <v>2.1056614418825545E-2</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="J19" s="33" cm="1">
         <f t="array" ref="J19">_xll.qlYieldTermStructureZeroRate($C$14,I19,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0887495689523087E-2</v>
+        <v>2.1804311905509664E-2</v>
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="J20" s="33" cm="1">
         <f t="array" ref="J20">_xll.qlYieldTermStructureZeroRate($C$14,I20,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1726812502017925E-2</v>
+        <v>2.3305383398994673E-2</v>
       </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="J21" s="33" cm="1">
         <f t="array" ref="J21">_xll.qlYieldTermStructureZeroRate($C$14,I21,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.2679838432030707E-2</v>
+        <v>2.5394439430906784E-2</v>
       </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="J22" s="38" cm="1">
         <f t="array" ref="J22">_xll.qlYieldTermStructureZeroRate($C$14,I22,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.3070178835056691E-2</v>
+        <v>2.6618940661949898E-2</v>
       </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="J28" s="28" cm="1">
         <f t="array" ref="J28">_xll.qlYieldTermStructureZeroRate($C$30,I28,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1489716353363754E-2</v>
+        <v>2.1489715124367082E-2</v>
       </c>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="J29" s="33" cm="1">
         <f t="array" ref="J29">_xll.qlYieldTermStructureZeroRate($C$30,I29,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1547205464292937E-2</v>
+        <v>2.1547204844790901E-2</v>
       </c>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="J30" s="33" cm="1">
         <f t="array" ref="J30">_xll.qlYieldTermStructureZeroRate($C$30,I30,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1965880406632231E-2</v>
+        <v>2.1964582886470737E-2</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.25">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="J31" s="33" cm="1">
         <f t="array" ref="J31">_xll.qlYieldTermStructureZeroRate($C$30,I31,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.2571071833691652E-2</v>
+        <v>2.2568918764418931E-2</v>
       </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="J32" s="33" cm="1">
         <f t="array" ref="J32">_xll.qlYieldTermStructureZeroRate($C$30,I32,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.3297154635597544E-2</v>
+        <v>2.3294217587170939E-2</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="J33" s="33" cm="1">
         <f t="array" ref="J33">_xll.qlYieldTermStructureZeroRate($C$30,I33,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.3960508648398035E-2</v>
+        <v>2.3957140103980739E-2</v>
       </c>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="J34" s="33" cm="1">
         <f t="array" ref="J34">_xll.qlYieldTermStructureZeroRate($C$30,I34,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.5306776040472129E-2</v>
+        <v>2.5305364889382738E-2</v>
       </c>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="J35" s="33" cm="1">
         <f t="array" ref="J35">_xll.qlYieldTermStructureZeroRate($C$30,I35,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.7212618430077776E-2</v>
+        <v>2.7224289747691924E-2</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="J36" s="38" cm="1">
         <f t="array" ref="J36">_xll.qlYieldTermStructureZeroRate($C$30,I36,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.8239633631788694E-2</v>
+        <v>2.8266282940571708E-2</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="J43" s="33" cm="1">
         <f t="array" ref="J43">_xll.qlYieldTermStructureZeroRate($C$44,I43,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.6998169757845402E-2</v>
+        <v>3.6998167414587564E-2</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="J44" s="33" cm="1">
         <f t="array" ref="J44">_xll.qlYieldTermStructureZeroRate($C$44,I44,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.6350947076966657E-2</v>
+        <v>3.6350945887968909E-2</v>
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="J45" s="33" cm="1">
         <f t="array" ref="J45">_xll.qlYieldTermStructureZeroRate($C$44,I45,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.4626291513237539E-2</v>
+        <v>3.4626290911888569E-2</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="J46" s="33" cm="1">
         <f t="array" ref="J46">_xll.qlYieldTermStructureZeroRate($C$44,I46,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.2256655936068857E-2</v>
+        <v>3.2751768392570955E-2</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="J47" s="33" cm="1">
         <f t="array" ref="J47">_xll.qlYieldTermStructureZeroRate($C$44,I47,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1464068845243616E-2</v>
+        <v>3.2377367024610644E-2</v>
       </c>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="J48" s="33" cm="1">
         <f t="array" ref="J48">_xll.qlYieldTermStructureZeroRate($C$44,I48,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1242194026496625E-2</v>
+        <v>3.2661635352545959E-2</v>
       </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="J49" s="33" cm="1">
         <f t="array" ref="J49">_xll.qlYieldTermStructureZeroRate($C$44,I49,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1174868169091315E-2</v>
+        <v>3.3148897734764607E-2</v>
       </c>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="J50" s="33" cm="1">
         <f t="array" ref="J50">_xll.qlYieldTermStructureZeroRate($C$44,I50,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1207428136625949E-2</v>
+        <v>3.4367701312975452E-2</v>
       </c>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="J51" s="33" cm="1">
         <f t="array" ref="J51">_xll.qlYieldTermStructureZeroRate($C$44,I51,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1186666702453285E-2</v>
+        <v>3.6219561600085722E-2</v>
       </c>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="J52" s="38" cm="1">
         <f t="array" ref="J52">_xll.qlYieldTermStructureZeroRate($C$44,I52,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1052022548249434E-2</v>
+        <v>3.7390996111162984E-2</v>
       </c>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
@@ -2426,15 +2426,15 @@
       </c>
       <c r="J58" s="28" cm="1">
         <f t="array" ref="J58">_xll.qlYieldTermStructureZeroRate($C$73,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9057055854570671E-2</v>
+        <v>1.9056934878278965E-2</v>
       </c>
       <c r="L58" s="28" cm="1">
         <f t="array" ref="L58">_xll.qlYieldTermStructureZeroRate($C$14,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.942332976750076E-2</v>
+        <v>1.9423329540682495E-2</v>
       </c>
       <c r="M58" s="49">
         <f>J58-L58</f>
-        <v>-3.6627391293008946E-4</v>
+        <v>-3.6639466240353039E-4</v>
       </c>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
@@ -2460,15 +2460,15 @@
       </c>
       <c r="J59" s="33" cm="1">
         <f t="array" ref="J59">_xll.qlYieldTermStructureZeroRate($C$73,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9150498713749881E-2</v>
+        <v>1.9341237502176117E-2</v>
       </c>
       <c r="L59" s="33" cm="1">
         <f t="array" ref="L59">_xll.qlYieldTermStructureZeroRate($C$14,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9516571239144988E-2</v>
+        <v>1.9707419970420838E-2</v>
       </c>
       <c r="M59" s="50">
-        <f t="shared" ref="M59:M65" si="0">J59-L59</f>
-        <v>-3.660725253951079E-4</v>
+        <f>J59-L59</f>
+        <v>-3.6618246824472039E-4</v>
       </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
@@ -2494,15 +2494,15 @@
       </c>
       <c r="J60" s="33" cm="1">
         <f t="array" ref="J60">_xll.qlYieldTermStructureZeroRate($C$73,I60,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9563249995868465E-2</v>
+        <v>1.9938542000702334E-2</v>
       </c>
       <c r="L60" s="33" cm="1">
         <f t="array" ref="L60">_xll.qlYieldTermStructureZeroRate($C$14,I60,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>1.9929171494420136E-2</v>
+        <v>2.0304501541429942E-2</v>
       </c>
       <c r="M60" s="50">
-        <f t="shared" si="0"/>
-        <v>-3.6592149855167039E-4</v>
+        <f>J60-L60</f>
+        <v>-3.6595954072760756E-4</v>
       </c>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
@@ -2529,15 +2529,15 @@
       </c>
       <c r="J61" s="33" cm="1">
         <f t="array" ref="J61">_xll.qlYieldTermStructureZeroRate($C$73,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0064553988159092E-2</v>
+        <v>2.0690783526765087E-2</v>
       </c>
       <c r="L61" s="33" cm="1">
         <f t="array" ref="L61">_xll.qlYieldTermStructureZeroRate($C$14,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0430384737421706E-2</v>
+        <v>2.1056614418825545E-2</v>
       </c>
       <c r="M61" s="50">
-        <f t="shared" si="0"/>
-        <v>-3.6583074926261477E-4</v>
+        <f>J61-L61</f>
+        <v>-3.6583089206045777E-4</v>
       </c>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
@@ -2564,15 +2564,15 @@
       </c>
       <c r="J62" s="33" cm="1">
         <f t="array" ref="J62">_xll.qlYieldTermStructureZeroRate($C$73,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0521737704570147E-2</v>
+        <v>2.1438592526394247E-2</v>
       </c>
       <c r="L62" s="33" cm="1">
         <f t="array" ref="L62">_xll.qlYieldTermStructureZeroRate($C$14,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.0887495689523087E-2</v>
+        <v>2.1804311905509664E-2</v>
       </c>
       <c r="M62" s="50">
-        <f t="shared" si="0"/>
-        <v>-3.6575798495293993E-4</v>
+        <f>J62-L62</f>
+        <v>-3.657193791154166E-4</v>
       </c>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
@@ -2599,15 +2599,15 @@
       </c>
       <c r="J63" s="33" cm="1">
         <f t="array" ref="J63">_xll.qlYieldTermStructureZeroRate($C$73,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1361165883865614E-2</v>
+        <v>2.2939847920213422E-2</v>
       </c>
       <c r="L63" s="33" cm="1">
         <f t="array" ref="L63">_xll.qlYieldTermStructureZeroRate($C$14,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.1726812502017925E-2</v>
+        <v>2.3305383398994673E-2</v>
       </c>
       <c r="M63" s="50">
-        <f t="shared" si="0"/>
-        <v>-3.6564661815231131E-4</v>
+        <f>J63-L63</f>
+        <v>-3.6553547878125092E-4</v>
       </c>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
@@ -2633,15 +2633,15 @@
       </c>
       <c r="J64" s="33" cm="1">
         <f t="array" ref="J64">_xll.qlYieldTermStructureZeroRate($C$73,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.2314305954994233E-2</v>
+        <v>2.5029132269805833E-2</v>
       </c>
       <c r="L64" s="33" cm="1">
         <f t="array" ref="L64">_xll.qlYieldTermStructureZeroRate($C$14,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.2679838432030707E-2</v>
+        <v>2.5394439430906784E-2</v>
       </c>
       <c r="M64" s="50">
-        <f t="shared" si="0"/>
-        <v>-3.6553247703647457E-4</v>
+        <f>J64-L64</f>
+        <v>-3.6530716110095077E-4</v>
       </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
@@ -2667,15 +2667,15 @@
       </c>
       <c r="J65" s="38" cm="1">
         <f t="array" ref="J65">_xll.qlYieldTermStructureZeroRate($C$73,I65,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.270469184326656E-2</v>
+        <v>2.6253758750164394E-2</v>
       </c>
       <c r="L65" s="38" cm="1">
         <f t="array" ref="L65">_xll.qlYieldTermStructureZeroRate($C$14,I65,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>2.3070178835056691E-2</v>
+        <v>2.6618940661949898E-2</v>
       </c>
       <c r="M65" s="51">
-        <f t="shared" si="0"/>
-        <v>-3.6548699179013086E-4</v>
+        <f>J65-L65</f>
+        <v>-3.6518191178550388E-4</v>
       </c>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
@@ -2773,11 +2773,11 @@
       </c>
       <c r="F79" s="56" cm="1">
         <f t="array" ref="F79">_xll.qlYieldTermStructureZeroRate($C$44,E79,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.7513671016082807E-2</v>
+        <v>3.7513715269406556E-2</v>
       </c>
       <c r="G79" s="49">
         <f>F79-M58</f>
-        <v>3.7879944929012893E-2</v>
+        <v>3.7880109931810083E-2</v>
       </c>
     </row>
     <row r="80" spans="2:13" x14ac:dyDescent="0.25">
@@ -2788,16 +2788,16 @@
         <v>27</v>
       </c>
       <c r="E80" s="57">
-        <f t="shared" ref="E80:E87" si="1">I58</f>
+        <f>I58</f>
         <v>46541</v>
       </c>
       <c r="F80" s="58" cm="1">
         <f t="array" ref="F80">_xll.qlYieldTermStructureZeroRate($C$44,E80,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.4626291513237539E-2</v>
+        <v>3.4626290911888569E-2</v>
       </c>
       <c r="G80" s="50">
-        <f t="shared" ref="G80:G87" si="2">F80-M58</f>
-        <v>3.4992565426167632E-2</v>
+        <f>F80-M58</f>
+        <v>3.4992685574292096E-2</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.25">
@@ -2809,100 +2809,100 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R81C3YieldTermStructureHandle,A</v>
       </c>
       <c r="E81" s="57">
-        <f t="shared" si="1"/>
+        <f>I59</f>
         <v>46909</v>
       </c>
       <c r="F81" s="58" cm="1">
         <f t="array" ref="F81">_xll.qlYieldTermStructureZeroRate($C$44,E81,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.2256655936068857E-2</v>
+        <v>3.2751768392570955E-2</v>
       </c>
       <c r="G81" s="50">
-        <f t="shared" si="2"/>
-        <v>3.2622728461463968E-2</v>
+        <f>F81-M59</f>
+        <v>3.3117950860815676E-2</v>
       </c>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E82" s="57">
-        <f t="shared" si="1"/>
+        <f>I60</f>
         <v>47273</v>
       </c>
       <c r="F82" s="58" cm="1">
         <f t="array" ref="F82">_xll.qlYieldTermStructureZeroRate($C$44,E82,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1464068845243616E-2</v>
+        <v>3.2377367024610644E-2</v>
       </c>
       <c r="G82" s="50">
-        <f t="shared" si="2"/>
-        <v>3.1829990343795286E-2</v>
+        <f>F82-M60</f>
+        <v>3.2743326565338252E-2</v>
       </c>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E83" s="57">
-        <f t="shared" si="1"/>
+        <f>I61</f>
         <v>47637</v>
       </c>
       <c r="F83" s="58" cm="1">
         <f t="array" ref="F83">_xll.qlYieldTermStructureZeroRate($C$44,E83,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1242194026496625E-2</v>
+        <v>3.2661635352545959E-2</v>
       </c>
       <c r="G83" s="50">
-        <f t="shared" si="2"/>
-        <v>3.160802477575924E-2</v>
+        <f>F83-M61</f>
+        <v>3.3027466244606417E-2</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E84" s="57">
-        <f t="shared" si="1"/>
+        <f>I62</f>
         <v>48002</v>
       </c>
       <c r="F84" s="58" cm="1">
         <f t="array" ref="F84">_xll.qlYieldTermStructureZeroRate($C$44,E84,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1174868169091315E-2</v>
+        <v>3.3148897734764607E-2</v>
       </c>
       <c r="G84" s="50">
-        <f t="shared" si="2"/>
-        <v>3.1540626154044252E-2</v>
+        <f>F84-M62</f>
+        <v>3.3514617113880027E-2</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E85" s="57">
-        <f t="shared" si="1"/>
+        <f>I63</f>
         <v>48733</v>
       </c>
       <c r="F85" s="58" cm="1">
         <f t="array" ref="F85">_xll.qlYieldTermStructureZeroRate($C$44,E85,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1207428136625949E-2</v>
+        <v>3.4367701312975452E-2</v>
       </c>
       <c r="G85" s="50">
-        <f t="shared" si="2"/>
-        <v>3.157307475477826E-2</v>
+        <f>F85-M63</f>
+        <v>3.4733236791756703E-2</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E86" s="57">
-        <f t="shared" si="1"/>
+        <f>I64</f>
         <v>49829</v>
       </c>
       <c r="F86" s="58" cm="1">
         <f t="array" ref="F86">_xll.qlYieldTermStructureZeroRate($C$44,E86,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1186666702453285E-2</v>
+        <v>3.6219561600085722E-2</v>
       </c>
       <c r="G86" s="50">
-        <f t="shared" si="2"/>
-        <v>3.1552199179489759E-2</v>
+        <f>F86-M64</f>
+        <v>3.6584868761186676E-2</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E87" s="59">
-        <f t="shared" si="1"/>
+        <f>I65</f>
         <v>50559</v>
       </c>
       <c r="F87" s="60" cm="1">
         <f t="array" ref="F87">_xll.qlYieldTermStructureZeroRate($C$44,E87,"Act/365","Continuous","NoFrequency",TRUE)</f>
-        <v>3.1052022548249434E-2</v>
+        <v>3.7390996111162984E-2</v>
       </c>
       <c r="G87" s="51">
-        <f t="shared" si="2"/>
-        <v>3.1417509540039565E-2</v>
+        <f>F87-M65</f>
+        <v>3.7756178022948492E-2</v>
       </c>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.25">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="C15" s="26" t="str" cm="1">
         <f t="array" ref="C15">_xll.xloRef(_xll.qlFixedRateLeg(C8,"30/360",10000,3%))</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R15C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R15C3,A</v>
       </c>
       <c r="G15" s="2">
         <v>49436</v>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C16" s="36" t="str" cm="1">
         <f t="array" ref="C16">_xll.xloRef(_xll.qlIborLeg(10000,C9,C11,"Act/360",,,,,,,,C12))</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3,A</v>
       </c>
       <c r="G16" s="2">
         <v>49800</v>
@@ -3422,7 +3422,7 @@
         <v>79</v>
       </c>
       <c r="C21" s="36" t="str" cm="1">
-        <f t="array" ref="C21">_xll.qlDiscountingSwapEngine(C20,,,,C2)</f>
+        <f t="array" ref="C21">_xll.qlDiscountingSwapEngine(C20,FALSE,,,C2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R21C3DiscountingSwapEngine,A</v>
       </c>
       <c r="G21" s="2" cm="1">
@@ -3471,10 +3471,10 @@
         <v>46512</v>
       </c>
       <c r="K22" s="9">
-        <v>2.138455344700926E-2</v>
+        <v>2.1384673222544164E-2</v>
       </c>
       <c r="L22" s="9">
-        <v>2.138455344700926E-2</v>
+        <v>2.1384673222544164E-2</v>
       </c>
       <c r="M22" s="10" t="str">
         <v>Actual/360</v>
@@ -3486,7 +3486,7 @@
         <v>10000</v>
       </c>
       <c r="P22" s="15">
-        <v>107.51678260857433</v>
+        <v>107.51738481334705</v>
       </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="C23" s="67" cm="1">
         <f t="array" ref="C23">_xll.qlInstrumentNPV(C18,_xll.qlInstrumentSetPricingEngine(C18,C21))</f>
-        <v>-245.62381627633476</v>
+        <v>-457.45759571020835</v>
       </c>
       <c r="G23" s="2">
         <v>46696</v>
@@ -3510,10 +3510,10 @@
         <v>46696</v>
       </c>
       <c r="K23" s="9">
-        <v>2.1806975526274315E-2</v>
+        <v>2.1805406705466268E-2</v>
       </c>
       <c r="L23" s="9">
-        <v>2.1806975526274315E-2</v>
+        <v>2.1805406705466268E-2</v>
       </c>
       <c r="M23" s="10" t="str">
         <v>Actual/360</v>
@@ -3525,7 +3525,7 @@
         <v>10000</v>
       </c>
       <c r="P23" s="15">
-        <v>111.45787491206872</v>
+        <v>111.44985649460537</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
@@ -3542,10 +3542,10 @@
         <v>46878</v>
       </c>
       <c r="K24" s="9">
-        <v>2.2401548096192391E-2</v>
+        <v>2.2398412231184286E-2</v>
       </c>
       <c r="L24" s="9">
-        <v>2.2401548096192391E-2</v>
+        <v>2.2398412231184286E-2</v>
       </c>
       <c r="M24" s="10" t="str">
         <v>Actual/360</v>
@@ -3557,7 +3557,7 @@
         <v>10000</v>
       </c>
       <c r="P24" s="15">
-        <v>113.25227093075041</v>
+        <v>113.23641739098721</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -3574,10 +3574,10 @@
         <v>47063</v>
       </c>
       <c r="K25" s="9">
-        <v>2.307390083860782E-2</v>
+        <v>2.3070332940635943E-2</v>
       </c>
       <c r="L25" s="9">
-        <v>2.307390083860782E-2</v>
+        <v>2.3070332940635943E-2</v>
       </c>
       <c r="M25" s="10" t="str">
         <v>Actual/360</v>
@@ -3589,7 +3589,7 @@
         <v>10000</v>
       </c>
       <c r="P25" s="15">
-        <v>118.57421264284574</v>
+        <v>118.55587761160136</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
@@ -3609,10 +3609,10 @@
         <v>47245</v>
       </c>
       <c r="K26" s="9">
-        <v>2.388421114349009E-2</v>
+        <v>2.3880186236089757E-2</v>
       </c>
       <c r="L26" s="9">
-        <v>2.388421114349009E-2</v>
+        <v>2.3880186236089757E-2</v>
       </c>
       <c r="M26" s="10" t="str">
         <v>Actual/360</v>
@@ -3624,7 +3624,7 @@
         <v>10000</v>
       </c>
       <c r="P26" s="15">
-        <v>120.74795633653324</v>
+        <v>120.72760819356488</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
@@ -3641,10 +3641,10 @@
         <v>47427</v>
       </c>
       <c r="K27" s="9">
-        <v>2.4812909407946986E-2</v>
+        <v>2.4808029409083519E-2</v>
       </c>
       <c r="L27" s="9">
-        <v>2.4812909407946986E-2</v>
+        <v>2.4808029409083519E-2</v>
       </c>
       <c r="M27" s="10" t="str">
         <v>Actual/360</v>
@@ -3656,7 +3656,7 @@
         <v>10000</v>
       </c>
       <c r="P27" s="15">
-        <v>125.44304200684309</v>
+        <v>125.41837090147779</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
@@ -3679,10 +3679,10 @@
         <v>47609</v>
       </c>
       <c r="K28" s="9">
-        <v>2.5564396707615327E-2</v>
+        <v>2.5558868460551245E-2</v>
       </c>
       <c r="L28" s="9">
-        <v>2.5564396707615327E-2</v>
+        <v>2.5558868460551245E-2</v>
       </c>
       <c r="M28" s="10" t="str">
         <v>Actual/360</v>
@@ -3694,7 +3694,7 @@
         <v>10000</v>
       </c>
       <c r="P28" s="15">
-        <v>129.24222779961082</v>
+        <v>129.21427943945352</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
@@ -3717,10 +3717,10 @@
         <v>47792</v>
       </c>
       <c r="K29" s="9">
-        <v>2.6069318165817593E-2</v>
+        <v>2.6063659195415808E-2</v>
       </c>
       <c r="L29" s="9">
-        <v>2.6069318165817593E-2</v>
+        <v>2.6063659195415808E-2</v>
       </c>
       <c r="M29" s="10" t="str">
         <v>Actual/360</v>
@@ -3732,7 +3732,7 @@
         <v>10000</v>
       </c>
       <c r="P29" s="15">
-        <v>132.51903400957278</v>
+        <v>132.49026757669702</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
@@ -3755,10 +3755,10 @@
         <v>47973</v>
       </c>
       <c r="K30" s="9">
-        <v>2.6616743283220688E-2</v>
+        <v>2.6611923626807494E-2</v>
       </c>
       <c r="L30" s="9">
-        <v>2.6616743283220688E-2</v>
+        <v>2.6611923626807494E-2</v>
       </c>
       <c r="M30" s="10" t="str">
         <v>Actual/360</v>
@@ -3770,7 +3770,7 @@
         <v>10000</v>
       </c>
       <c r="P30" s="15">
-        <v>133.82307039619289</v>
+        <v>133.79883823478212</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
@@ -3794,10 +3794,10 @@
         <v>48157</v>
       </c>
       <c r="K31" s="9">
-        <v>2.7315692011382765E-2</v>
+        <v>2.7312856251532784E-2</v>
       </c>
       <c r="L31" s="9">
-        <v>2.7315692011382765E-2</v>
+        <v>2.7312856251532784E-2</v>
       </c>
       <c r="M31" s="10" t="str">
         <v>Actual/360</v>
@@ -3809,7 +3809,7 @@
         <v>10000</v>
       </c>
       <c r="P31" s="15">
-        <v>139.61353694706747</v>
+        <v>139.59904306338979</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
@@ -3833,10 +3833,10 @@
         <v>48339</v>
       </c>
       <c r="K32" s="9">
-        <v>2.8036965686711039E-2</v>
+        <v>2.803720508332961E-2</v>
       </c>
       <c r="L32" s="9">
-        <v>2.8036965686711039E-2</v>
+        <v>2.803720508332961E-2</v>
       </c>
       <c r="M32" s="10" t="str">
         <v>Actual/360</v>
@@ -3848,7 +3848,7 @@
         <v>10000</v>
       </c>
       <c r="P32" s="15">
-        <v>141.74243763837245</v>
+        <v>141.74364792127747</v>
       </c>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.25">
@@ -3872,10 +3872,10 @@
         <v>48523</v>
       </c>
       <c r="K33" s="9">
-        <v>2.8740748622150356E-2</v>
+        <v>2.8745130540238736E-2</v>
       </c>
       <c r="L33" s="9">
-        <v>2.8740748622150356E-2</v>
+        <v>2.8745130540238736E-2</v>
       </c>
       <c r="M33" s="10" t="str">
         <v>Actual/360</v>
@@ -3887,7 +3887,7 @@
         <v>10000</v>
       </c>
       <c r="P33" s="15">
-        <v>146.89715962432405</v>
+        <v>146.91955609455354</v>
       </c>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
@@ -3904,10 +3904,10 @@
         <v>48704</v>
       </c>
       <c r="K34" s="9">
-        <v>2.9415049697704677E-2</v>
+        <v>2.9424619959732837E-2</v>
       </c>
       <c r="L34" s="9">
-        <v>2.9415049697704677E-2</v>
+        <v>2.9424619959732837E-2</v>
       </c>
       <c r="M34" s="10" t="str">
         <v>Actual/360</v>
@@ -3919,7 +3919,7 @@
         <v>10000</v>
       </c>
       <c r="P34" s="15">
-        <v>147.89233320234851</v>
+        <v>147.94045035310123</v>
       </c>
     </row>
     <row r="35" spans="2:16" x14ac:dyDescent="0.25">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="C35" s="45" t="str" cm="1">
         <f t="array" ref="C35">_xll.xloRef(C37:C56)</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R35C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Euribor swap!R35C3,A</v>
       </c>
       <c r="G35" s="2">
         <v>48890</v>
@@ -3943,10 +3943,10 @@
         <v>48890</v>
       </c>
       <c r="K35" s="9">
-        <v>3.0077170146981556E-2</v>
+        <v>3.0093093110223252E-2</v>
       </c>
       <c r="L35" s="9">
-        <v>3.0077170146981556E-2</v>
+        <v>3.0093093110223252E-2</v>
       </c>
       <c r="M35" s="10" t="str">
         <v>Actual/360</v>
@@ -3958,7 +3958,7 @@
         <v>10000</v>
       </c>
       <c r="P35" s="15">
-        <v>155.3987124260714</v>
+        <v>155.48098106948683</v>
       </c>
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.25">
@@ -3975,10 +3975,10 @@
         <v>49069</v>
       </c>
       <c r="K36" s="9">
-        <v>3.0674042823818502E-2</v>
+        <v>3.069771615578586E-2</v>
       </c>
       <c r="L36" s="9">
-        <v>3.0674042823818502E-2</v>
+        <v>3.069771615578586E-2</v>
       </c>
       <c r="M36" s="10" t="str">
         <v>Actual/360</v>
@@ -3990,7 +3990,7 @@
         <v>10000</v>
       </c>
       <c r="P36" s="15">
-        <v>152.51815737398644</v>
+        <v>152.63586644126858</v>
       </c>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.25">
@@ -4015,10 +4015,10 @@
         <v>49254</v>
       </c>
       <c r="K37" s="9">
-        <v>3.1230840498327264E-2</v>
+        <v>3.1263858466951552E-2</v>
       </c>
       <c r="L37" s="9">
-        <v>3.1230840498327264E-2</v>
+        <v>3.1263858466951552E-2</v>
       </c>
       <c r="M37" s="10" t="str">
         <v>Actual/360</v>
@@ -4030,7 +4030,7 @@
         <v>10000</v>
       </c>
       <c r="P37" s="15">
-        <v>160.49181922751509</v>
+        <v>160.66149489961214</v>
       </c>
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.25">
@@ -4054,10 +4054,10 @@
         <v>49436</v>
       </c>
       <c r="K38" s="9">
-        <v>3.1724801684909702E-2</v>
+        <v>3.1768810222157939E-2</v>
       </c>
       <c r="L38" s="9">
-        <v>3.1724801684909702E-2</v>
+        <v>3.1768810222157939E-2</v>
       </c>
       <c r="M38" s="10" t="str">
         <v>Actual/360</v>
@@ -4069,7 +4069,7 @@
         <v>10000</v>
       </c>
       <c r="P38" s="15">
-        <v>160.38649740704346</v>
+        <v>160.6089850120207</v>
       </c>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.25">
@@ -4093,10 +4093,10 @@
         <v>49618</v>
       </c>
       <c r="K39" s="9">
-        <v>3.2163468565114643E-2</v>
+        <v>3.2219974315495802E-2</v>
       </c>
       <c r="L39" s="9">
-        <v>3.2163468565114643E-2</v>
+        <v>3.2219974315495802E-2</v>
       </c>
       <c r="M39" s="10" t="str">
         <v>Actual/360</v>
@@ -4108,7 +4108,7 @@
         <v>10000</v>
       </c>
       <c r="P39" s="15">
-        <v>162.60420219030181</v>
+        <v>162.8898701505621</v>
       </c>
     </row>
     <row r="40" spans="2:16" x14ac:dyDescent="0.25">
@@ -4132,10 +4132,10 @@
         <v>49800</v>
       </c>
       <c r="K40" s="9">
-        <v>3.2547135883612875E-2</v>
+        <v>3.2617718239904392E-2</v>
       </c>
       <c r="L40" s="9">
-        <v>3.2547135883612875E-2</v>
+        <v>3.2617718239904392E-2</v>
       </c>
       <c r="M40" s="10" t="str">
         <v>Actual/360</v>
@@ -4147,7 +4147,7 @@
         <v>10000</v>
       </c>
       <c r="P40" s="15">
-        <v>164.54385363382062</v>
+        <v>164.90068665729441</v>
       </c>
     </row>
     <row r="41" spans="2:16" x14ac:dyDescent="0.25">
@@ -4280,10 +4280,10 @@
         <v>46512</v>
       </c>
       <c r="K46" s="9">
-        <v>2.138455344700926E-2</v>
+        <v>2.1384673222544164E-2</v>
       </c>
       <c r="L46" s="9">
-        <v>2.1277660362714525E-2</v>
+        <v>2.127777424199288E-2</v>
       </c>
       <c r="M46" s="10" t="str">
         <v>Actual/360</v>
@@ -4295,7 +4295,7 @@
         <v>10000</v>
       </c>
       <c r="P46" s="15">
-        <v>106.97934793475915</v>
+        <v>106.9799204944642</v>
       </c>
     </row>
     <row r="47" spans="2:16" x14ac:dyDescent="0.25">
@@ -4319,10 +4319,10 @@
         <v>46696</v>
       </c>
       <c r="K47" s="9">
-        <v>2.1806975526274315E-2</v>
+        <v>2.1805406705466268E-2</v>
       </c>
       <c r="L47" s="9">
-        <v>2.1250528373199712E-2</v>
+        <v>2.1249187218489684E-2</v>
       </c>
       <c r="M47" s="10" t="str">
         <v>Actual/360</v>
@@ -4334,7 +4334,7 @@
         <v>10000</v>
       </c>
       <c r="P47" s="15">
-        <v>108.61381168524296</v>
+        <v>108.60695689450282</v>
       </c>
     </row>
     <row r="48" spans="2:16" x14ac:dyDescent="0.25">
@@ -4358,10 +4358,10 @@
         <v>46878</v>
       </c>
       <c r="K48" s="9">
-        <v>2.2401548096192391E-2</v>
+        <v>2.2398412231184286E-2</v>
       </c>
       <c r="L48" s="9">
-        <v>2.1275639186179626E-2</v>
+        <v>2.1273201147721705E-2</v>
       </c>
       <c r="M48" s="10" t="str">
         <v>Actual/360</v>
@@ -4373,7 +4373,7 @@
         <v>10000</v>
       </c>
       <c r="P48" s="15">
-        <v>107.56017588568588</v>
+        <v>107.54785024681529</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.25">
@@ -4397,10 +4397,10 @@
         <v>47063</v>
       </c>
       <c r="K49" s="9">
-        <v>2.307390083860782E-2</v>
+        <v>2.3070332940635943E-2</v>
       </c>
       <c r="L49" s="9">
-        <v>2.1351204123283209E-2</v>
+        <v>2.1348652906788473E-2</v>
       </c>
       <c r="M49" s="10" t="str">
         <v>Actual/360</v>
@@ -4412,7 +4412,7 @@
         <v>10000</v>
       </c>
       <c r="P49" s="15">
-        <v>109.72146563353871</v>
+        <v>109.70835521544075</v>
       </c>
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.25">
@@ -4436,10 +4436,10 @@
         <v>47245</v>
       </c>
       <c r="K50" s="9">
-        <v>2.388421114349009E-2</v>
+        <v>2.3880186236089757E-2</v>
       </c>
       <c r="L50" s="9">
-        <v>2.1516914919894454E-2</v>
+        <v>2.1514255592564761E-2</v>
       </c>
       <c r="M50" s="10" t="str">
         <v>Actual/360</v>
@@ -4451,7 +4451,7 @@
         <v>10000</v>
       </c>
       <c r="P50" s="15">
-        <v>108.77995876168863</v>
+        <v>108.76651438463294</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
@@ -4475,10 +4475,10 @@
         <v>47427</v>
       </c>
       <c r="K51" s="9">
-        <v>2.4819275330840575E-2</v>
+        <v>2.4814390296047376E-2</v>
       </c>
       <c r="L51" s="9">
-        <v>2.1750400688391403E-2</v>
+        <v>2.1747409452571989E-2</v>
       </c>
       <c r="M51" s="10" t="str">
         <v>Actual/360</v>
@@ -4490,7 +4490,7 @@
         <v>10000</v>
       </c>
       <c r="P51" s="15">
-        <v>109.96035903575653</v>
+        <v>109.94523667689172</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.25">
@@ -4514,10 +4514,10 @@
         <v>47609</v>
       </c>
       <c r="K52" s="9">
-        <v>2.5564396707615327E-2</v>
+        <v>2.5558868460551245E-2</v>
       </c>
       <c r="L52" s="9">
-        <v>2.186816613206613E-2</v>
+        <v>2.1864982852607934E-2</v>
       </c>
       <c r="M52" s="10" t="str">
         <v>Actual/360</v>
@@ -4529,7 +4529,7 @@
         <v>10000</v>
       </c>
       <c r="P52" s="15">
-        <v>110.55572877877876</v>
+        <v>110.53963553262899</v>
       </c>
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.25">
@@ -4553,10 +4553,10 @@
         <v>47792</v>
       </c>
       <c r="K53" s="9">
-        <v>2.6071620365621651E-2</v>
+        <v>2.6065962255220138E-2</v>
       </c>
       <c r="L53" s="9">
-        <v>2.1851960968941261E-2</v>
+        <v>2.1848859102225452E-2</v>
       </c>
       <c r="M53" s="10" t="str">
         <v>Actual/360</v>
@@ -4568,7 +4568,7 @@
         <v>10000</v>
       </c>
       <c r="P53" s="15">
-        <v>111.08080159211806</v>
+        <v>111.06503376964604</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.25">
@@ -4592,10 +4592,10 @@
         <v>47973</v>
       </c>
       <c r="K54" s="9">
-        <v>2.6616743283220688E-2</v>
+        <v>2.6611923626807494E-2</v>
       </c>
       <c r="L54" s="9">
-        <v>2.1869529716103349E-2</v>
+        <v>2.1867009364734496E-2</v>
       </c>
       <c r="M54" s="10" t="str">
         <v>Actual/360</v>
@@ -4607,7 +4607,7 @@
         <v>10000</v>
       </c>
       <c r="P54" s="15">
-        <v>109.95513551707516</v>
+        <v>109.94246375047065</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.25">
@@ -4631,10 +4631,10 @@
         <v>48157</v>
       </c>
       <c r="K55" s="9">
-        <v>2.7315692011382765E-2</v>
+        <v>2.7312856251532784E-2</v>
       </c>
       <c r="L55" s="9">
-        <v>2.1975383807419716E-2</v>
+        <v>2.1973970444877509E-2</v>
       </c>
       <c r="M55" s="10" t="str">
         <v>Actual/360</v>
@@ -4646,7 +4646,7 @@
         <v>10000</v>
       </c>
       <c r="P55" s="15">
-        <v>112.31862834903409</v>
+        <v>112.31140449604059</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.25">
@@ -4670,10 +4670,10 @@
         <v>48339</v>
       </c>
       <c r="K56" s="9">
-        <v>2.8036965686711039E-2</v>
+        <v>2.803720508332961E-2</v>
       </c>
       <c r="L56" s="9">
-        <v>2.2082848383185427E-2</v>
+        <v>2.2082962262496796E-2</v>
       </c>
       <c r="M56" s="10" t="str">
         <v>Actual/360</v>
@@ -4685,7 +4685,7 @@
         <v>10000</v>
       </c>
       <c r="P56" s="15">
-        <v>111.64106682610409</v>
+        <v>111.64164254928934</v>
       </c>
     </row>
     <row r="57" spans="2:16" x14ac:dyDescent="0.25">
@@ -4702,10 +4702,10 @@
         <v>48523</v>
       </c>
       <c r="K57" s="9">
-        <v>2.8740748622150356E-2</v>
+        <v>2.8745130540238736E-2</v>
       </c>
       <c r="L57" s="9">
-        <v>2.2187819608281735E-2</v>
+        <v>2.2189816662577588E-2</v>
       </c>
       <c r="M57" s="10" t="str">
         <v>Actual/360</v>
@@ -4717,7 +4717,7 @@
         <v>10000</v>
       </c>
       <c r="P57" s="15">
-        <v>113.40441133121776</v>
+        <v>113.41461849761878</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.25">
@@ -4734,10 +4734,10 @@
         <v>48704</v>
       </c>
       <c r="K58" s="9">
-        <v>2.9415049697704677E-2</v>
+        <v>2.9424619959732837E-2</v>
       </c>
       <c r="L58" s="9">
-        <v>2.2276794557951701E-2</v>
+        <v>2.2280985491747663E-2</v>
       </c>
       <c r="M58" s="10" t="str">
         <v>Actual/360</v>
@@ -4749,7 +4749,7 @@
         <v>10000</v>
       </c>
       <c r="P58" s="15">
-        <v>112.00277263859049</v>
+        <v>112.02384372239797</v>
       </c>
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.25">
@@ -4766,10 +4766,10 @@
         <v>48890</v>
       </c>
       <c r="K59" s="9">
-        <v>3.0077170146981556E-2</v>
+        <v>3.0093093110223252E-2</v>
       </c>
       <c r="L59" s="9">
-        <v>2.2363929165041825E-2</v>
+        <v>2.2370646727096273E-2</v>
       </c>
       <c r="M59" s="10" t="str">
         <v>Actual/360</v>
@@ -4781,7 +4781,7 @@
         <v>10000</v>
       </c>
       <c r="P59" s="15">
-        <v>115.54696735271611</v>
+        <v>115.58167475666409</v>
       </c>
     </row>
     <row r="60" spans="2:16" x14ac:dyDescent="0.25">
@@ -4798,10 +4798,10 @@
         <v>49069</v>
       </c>
       <c r="K60" s="9">
-        <v>3.0682617909938158E-2</v>
+        <v>3.0706369802926844E-2</v>
       </c>
       <c r="L60" s="9">
-        <v>2.2421271049279663E-2</v>
+        <v>2.2430924263380836E-2</v>
       </c>
       <c r="M60" s="10" t="str">
         <v>Actual/360</v>
@@ -4813,7 +4813,7 @@
         <v>10000</v>
       </c>
       <c r="P60" s="15">
-        <v>111.48354216169611</v>
+        <v>111.53154008736583</v>
       </c>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.25">
@@ -4830,10 +4830,10 @@
         <v>49254</v>
       </c>
       <c r="K61" s="9">
-        <v>3.1230840498327264E-2</v>
+        <v>3.1263858466951552E-2</v>
       </c>
       <c r="L61" s="9">
-        <v>2.2467254576994548E-2</v>
+        <v>2.2480305060973024E-2</v>
       </c>
       <c r="M61" s="10" t="str">
         <v>Actual/360</v>
@@ -4845,7 +4845,7 @@
         <v>10000</v>
       </c>
       <c r="P61" s="15">
-        <v>115.45672490955532</v>
+        <v>115.52378989666693</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.25">
@@ -4862,10 +4862,10 @@
         <v>49436</v>
       </c>
       <c r="K62" s="9">
-        <v>3.1724801684909702E-2</v>
+        <v>3.1768810222157939E-2</v>
       </c>
       <c r="L62" s="9">
-        <v>2.2489148503597511E-2</v>
+        <v>2.250605686265305E-2</v>
       </c>
       <c r="M62" s="10" t="str">
         <v>Actual/360</v>
@@ -4877,7 +4877,7 @@
         <v>10000</v>
       </c>
       <c r="P62" s="15">
-        <v>113.6951396570763</v>
+        <v>113.78062080563485</v>
       </c>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.25">
@@ -4894,10 +4894,10 @@
         <v>49618</v>
       </c>
       <c r="K63" s="9">
-        <v>3.2168534895650386E-2</v>
+        <v>3.2225125163265818E-2</v>
       </c>
       <c r="L63" s="9">
-        <v>2.2494172754229883E-2</v>
+        <v>2.2515331732274785E-2</v>
       </c>
       <c r="M63" s="10" t="str">
         <v>Actual/360</v>
@@ -4909,7 +4909,7 @@
         <v>10000</v>
       </c>
       <c r="P63" s="15">
-        <v>113.72054003527329</v>
+        <v>113.82751042427807</v>
       </c>
     </row>
     <row r="64" spans="2:16" x14ac:dyDescent="0.25">
@@ -4926,10 +4926,10 @@
         <v>49800</v>
       </c>
       <c r="K64" s="9">
-        <v>3.2547135883612875E-2</v>
+        <v>3.2617718239904392E-2</v>
       </c>
       <c r="L64" s="9">
-        <v>2.248252921577935E-2</v>
+        <v>2.2508349557449091E-2</v>
       </c>
       <c r="M64" s="10" t="str">
         <v>Actual/360</v>
@@ -4941,7 +4941,7 @@
         <v>10000</v>
       </c>
       <c r="P64" s="15">
-        <v>113.66167547977336</v>
+        <v>113.79221165154817</v>
       </c>
     </row>
   </sheetData>
@@ -5042,10 +5042,10 @@
         <v>46239</v>
       </c>
       <c r="K7" s="9">
-        <v>3.6300457932529895E-2</v>
+        <v>3.6300892782605843E-2</v>
       </c>
       <c r="L7" s="9">
-        <v>3.6838204095413718E-2</v>
+        <v>3.6836333530602845E-2</v>
       </c>
       <c r="M7" s="10" t="str">
         <v>Actual/360</v>
@@ -5057,7 +5057,7 @@
         <v>10000</v>
       </c>
       <c r="P7" s="15">
-        <v>94.142077132723927</v>
+        <v>94.137296800429482</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
@@ -5081,10 +5081,10 @@
         <v>46331</v>
       </c>
       <c r="K8" s="9">
-        <v>3.4909402309519777E-2</v>
+        <v>3.4903267785271197E-2</v>
       </c>
       <c r="L8" s="9">
-        <v>3.5830529456076163E-2</v>
+        <v>3.5840395094037518E-2</v>
       </c>
       <c r="M8" s="10" t="str">
         <v>Actual/360</v>
@@ -5096,7 +5096,7 @@
         <v>10000</v>
       </c>
       <c r="P8" s="15">
-        <v>91.566908609972415</v>
+        <v>91.59212079587364</v>
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.25">
@@ -5114,10 +5114,10 @@
         <v>46423</v>
       </c>
       <c r="K9" s="9">
-        <v>3.2871520974318003E-2</v>
+        <v>3.2783761795753819E-2</v>
       </c>
       <c r="L9" s="9">
-        <v>3.4011836574586875E-2</v>
+        <v>3.3946514725718635E-2</v>
       </c>
       <c r="M9" s="10" t="str">
         <v>Actual/360</v>
@@ -5129,7 +5129,7 @@
         <v>10000</v>
       </c>
       <c r="P9" s="15">
-        <v>86.919137912833122</v>
+        <v>86.752204299058718</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.25">
@@ -5153,10 +5153,10 @@
         <v>46512</v>
       </c>
       <c r="K10" s="9">
-        <v>3.1318626551826156E-2</v>
+        <v>3.1446115407218755E-2</v>
       </c>
       <c r="L10" s="9">
-        <v>3.2171865192229157E-2</v>
+        <v>3.2166659726863438E-2</v>
       </c>
       <c r="M10" s="10" t="str">
         <v>Actual/360</v>
@@ -5168,7 +5168,7 @@
         <v>10000</v>
       </c>
       <c r="P10" s="15">
-        <v>79.536000058566543</v>
+        <v>79.523130991412387</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
@@ -5185,10 +5185,10 @@
         <v>46604</v>
       </c>
       <c r="K11" s="9">
-        <v>3.0185225830150486E-2</v>
+        <v>3.0764412892860804E-2</v>
       </c>
       <c r="L11" s="9">
-        <v>3.0832284063057869E-2</v>
+        <v>3.1190673870930337E-2</v>
       </c>
       <c r="M11" s="10" t="str">
         <v>Actual/360</v>
@@ -5200,7 +5200,7 @@
         <v>10000</v>
       </c>
       <c r="P11" s="15">
-        <v>78.793614827814551</v>
+        <v>79.709499892377522</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
@@ -5208,7 +5208,7 @@
         <v>92</v>
       </c>
       <c r="C12" s="26" t="str" cm="1">
-        <f t="array" ref="C12">_xll.qlOvernightIndexedSwap("Payer",10000,C8,0.03,"Act/360",C10,,,,,,,,,,C2)</f>
+        <f t="array" ref="C12">_xll.qlOvernightIndexedSwap("Payer",10000,C8,0.03,"Act/360",C10,0,0,"Following","TARGET",,,,,,C2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Sofr swap!R12C3OvernightIndexedSwap,A</v>
       </c>
       <c r="G12" s="2">
@@ -5224,10 +5224,10 @@
         <v>46696</v>
       </c>
       <c r="K12" s="9">
-        <v>2.9417431475335931E-2</v>
+        <v>3.0366288404684028E-2</v>
       </c>
       <c r="L12" s="9">
-        <v>2.9879647693866945E-2</v>
+        <v>3.0660331619406175E-2</v>
       </c>
       <c r="M12" s="10" t="str">
         <v>Actual/360</v>
@@ -5239,7 +5239,7 @@
         <v>10000</v>
       </c>
       <c r="P12" s="15">
-        <v>76.359099662104413</v>
+        <v>78.354180805149113</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="C13" s="31" t="str" cm="1">
         <f t="array" ref="C13">_xll.xloRef(_xll.qlSwapLeg(C12,0))</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R13C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R13C3,A</v>
       </c>
       <c r="G13" s="2">
         <v>46787</v>
@@ -5263,10 +5263,10 @@
         <v>46790</v>
       </c>
       <c r="K13" s="9">
-        <v>2.9006882292366143E-2</v>
+        <v>3.0223198656980088E-2</v>
       </c>
       <c r="L13" s="9">
-        <v>2.9286685335029195E-2</v>
+        <v>3.038929608565465E-2</v>
       </c>
       <c r="M13" s="10" t="str">
         <v>Actual/360</v>
@@ -5278,7 +5278,7 @@
         <v>10000</v>
       </c>
       <c r="P13" s="15">
-        <v>76.470789485909577</v>
+        <v>79.349828668098255</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="C14" s="36" t="str" cm="1">
         <f t="array" ref="C14">_xll.xloRef(_xll.qlSwapLeg(C12,1))</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R14C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R14C3,A</v>
       </c>
       <c r="G14" s="2">
         <v>46877</v>
@@ -5302,10 +5302,10 @@
         <v>46878</v>
       </c>
       <c r="K14" s="9">
-        <v>2.895136866986725E-2</v>
+        <v>3.0323062670332135E-2</v>
       </c>
       <c r="L14" s="9">
-        <v>2.9050687640267921E-2</v>
+        <v>3.0363955160805013E-2</v>
       </c>
       <c r="M14" s="10" t="str">
         <v>Actual/360</v>
@@ -5317,7 +5317,7 @@
         <v>10000</v>
       </c>
       <c r="P14" s="15">
-        <v>71.012792009543801</v>
+        <v>74.223001504190037</v>
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
@@ -5334,10 +5334,10 @@
         <v>46972</v>
       </c>
       <c r="K15" s="9">
-        <v>2.9172911154997649E-2</v>
+        <v>3.0641829466837578E-2</v>
       </c>
       <c r="L15" s="9">
-        <v>2.9165378776181083E-2</v>
+        <v>3.0595566745615754E-2</v>
       </c>
       <c r="M15" s="10" t="str">
         <v>Actual/360</v>
@@ -5349,7 +5349,7 @@
         <v>10000</v>
       </c>
       <c r="P15" s="15">
-        <v>76.154044582250606</v>
+        <v>79.888424280218914</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
@@ -5367,10 +5367,10 @@
         <v>47063</v>
       </c>
       <c r="K16" s="9">
-        <v>2.939639214023515E-2</v>
+        <v>3.1019752065493122E-2</v>
       </c>
       <c r="L16" s="9">
-        <v>2.9394434881040286E-2</v>
+        <v>3.0948769438463003E-2</v>
       </c>
       <c r="M16" s="10" t="str">
         <v>Actual/360</v>
@@ -5382,7 +5382,7 @@
         <v>10000</v>
       </c>
       <c r="P16" s="15">
-        <v>74.302599282629615</v>
+        <v>78.231611636114806</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
@@ -5403,10 +5403,10 @@
         <v>47154</v>
       </c>
       <c r="K17" s="9">
-        <v>2.9607774051756408E-2</v>
+        <v>3.1454393409502401E-2</v>
       </c>
       <c r="L17" s="9">
-        <v>2.9613233397121637E-2</v>
+        <v>3.1359086989368928E-2</v>
       </c>
       <c r="M17" s="10" t="str">
         <v>Actual/360</v>
@@ -5418,7 +5418,7 @@
         <v>10000</v>
       </c>
       <c r="P17" s="15">
-        <v>74.855673309390795</v>
+        <v>79.268803223127009</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
@@ -5436,10 +5436,10 @@
         <v>47245</v>
       </c>
       <c r="K18" s="9">
-        <v>2.9807056825692513E-2</v>
+        <v>3.1945754115012548E-2</v>
       </c>
       <c r="L18" s="9">
-        <v>2.9819856220898933E-2</v>
+        <v>3.1826605240600644E-2</v>
       </c>
       <c r="M18" s="10" t="str">
         <v>Actual/360</v>
@@ -5451,7 +5451,7 @@
         <v>10000</v>
       </c>
       <c r="P18" s="15">
-        <v>75.377969891716745</v>
+        <v>80.450585469296072</v>
       </c>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.25">
@@ -5475,10 +5475,10 @@
         <v>47336</v>
       </c>
       <c r="K19" s="9">
-        <v>2.9989261497656017E-2</v>
+        <v>3.2469903096137287E-2</v>
       </c>
       <c r="L19" s="9">
-        <v>3.0013087145352245E-2</v>
+        <v>3.2345504246838616E-2</v>
       </c>
       <c r="M19" s="10" t="str">
         <v>Actual/360</v>
@@ -5490,7 +5490,7 @@
         <v>10000</v>
       </c>
       <c r="P19" s="15">
-        <v>75.866414728529293</v>
+        <v>81.762246846175387</v>
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
@@ -5514,10 +5514,10 @@
         <v>47427</v>
       </c>
       <c r="K20" s="9">
-        <v>3.0138715543222006E-2</v>
+        <v>3.2951508805423302E-2</v>
       </c>
       <c r="L20" s="9">
-        <v>3.0180044291988437E-2</v>
+        <v>3.2853854285936783E-2</v>
       </c>
       <c r="M20" s="10" t="str">
         <v>Actual/360</v>
@@ -5529,7 +5529,7 @@
         <v>10000</v>
       </c>
       <c r="P20" s="15">
-        <v>76.288445293637437</v>
+        <v>83.047242778340191</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
@@ -5546,10 +5546,10 @@
         <v>47519</v>
       </c>
       <c r="K21" s="9">
-        <v>3.0253890321123578E-2</v>
+        <v>3.3390954298271325E-2</v>
       </c>
       <c r="L21" s="9">
-        <v>3.031484413256615E-2</v>
+        <v>3.3318223869135556E-2</v>
       </c>
       <c r="M21" s="10" t="str">
         <v>Actual/360</v>
@@ -5561,7 +5561,7 @@
         <v>10000</v>
       </c>
       <c r="P21" s="15">
-        <v>77.471268338780149</v>
+        <v>85.146572110013082</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
@@ -5584,10 +5584,10 @@
         <v>47609</v>
       </c>
       <c r="K22" s="9">
-        <v>3.0335932245817432E-2</v>
+        <v>3.3770558026322561E-2</v>
       </c>
       <c r="L22" s="9">
-        <v>3.0410941969284622E-2</v>
+        <v>3.3727014914982867E-2</v>
       </c>
       <c r="M22" s="10" t="str">
         <v>Actual/360</v>
@@ -5599,7 +5599,7 @@
         <v>10000</v>
       </c>
       <c r="P22" s="15">
-        <v>76.027354923211561</v>
+        <v>84.317537287457171</v>
       </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
@@ -5623,10 +5623,10 @@
         <v>47700</v>
       </c>
       <c r="K23" s="9">
-        <v>3.0393367377827829E-2</v>
+        <v>3.4122997817060963E-2</v>
       </c>
       <c r="L23" s="9">
-        <v>3.0478732812397782E-2</v>
+        <v>3.4093744179683562E-2</v>
       </c>
       <c r="M23" s="10" t="str">
         <v>Actual/360</v>
@@ -5638,7 +5638,7 @@
         <v>10000</v>
       </c>
       <c r="P23" s="15">
-        <v>77.043463498005508</v>
+        <v>86.181408898644563</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
@@ -5661,10 +5661,10 @@
         <v>47792</v>
       </c>
       <c r="K24" s="9">
-        <v>3.0455942067177943E-2</v>
+        <v>3.4494536317080104E-2</v>
       </c>
       <c r="L24" s="9">
-        <v>3.0540609519527088E-2</v>
+        <v>3.4458837480995486E-2</v>
       </c>
       <c r="M24" s="10" t="str">
         <v>Actual/360</v>
@@ -5676,7 +5676,7 @@
         <v>10000</v>
       </c>
       <c r="P24" s="15">
-        <v>78.04822432768033</v>
+        <v>88.061473562544009</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -5699,10 +5699,10 @@
         <v>47884</v>
       </c>
       <c r="K25" s="9">
-        <v>3.0529064077944312E-2</v>
+        <v>3.488336534965164E-2</v>
       </c>
       <c r="L25" s="9">
-        <v>3.0609993142381178E-2</v>
+        <v>3.4842097886160002E-2</v>
       </c>
       <c r="M25" s="10" t="str">
         <v>Actual/360</v>
@@ -5714,7 +5714,7 @@
         <v>10000</v>
       </c>
       <c r="P25" s="15">
-        <v>78.225538030529677</v>
+        <v>89.040916820186666</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
@@ -5737,10 +5737,10 @@
         <v>47973</v>
       </c>
       <c r="K26" s="9">
-        <v>3.0609689372731452E-2</v>
+        <v>3.5275577420232906E-2</v>
       </c>
       <c r="L26" s="9">
-        <v>3.0682800504072221E-2</v>
+        <v>3.5231646152900656E-2</v>
       </c>
       <c r="M26" s="10" t="str">
         <v>Actual/360</v>
@@ -5752,7 +5752,7 @@
         <v>10000</v>
       </c>
       <c r="P26" s="15">
-        <v>75.85470124617855</v>
+        <v>87.100458544671085</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
@@ -5775,10 +5775,10 @@
         <v>48065</v>
       </c>
       <c r="K27" s="9">
-        <v>3.0693367513121572E-2</v>
+        <v>3.5692789592243201E-2</v>
       </c>
       <c r="L27" s="9">
-        <v>3.0770789752441189E-2</v>
+        <v>3.5647322000486377E-2</v>
       </c>
       <c r="M27" s="10" t="str">
         <v>Actual/360</v>
@@ -5790,7 +5790,7 @@
         <v>10000</v>
       </c>
       <c r="P27" s="15">
-        <v>78.636462700683026</v>
+        <v>91.098711779020732</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
@@ -5813,10 +5813,10 @@
         <v>48157</v>
       </c>
       <c r="K28" s="9">
-        <v>3.0767778409206414E-2</v>
+        <v>3.6093794056197837E-2</v>
       </c>
       <c r="L28" s="9">
-        <v>3.0851651969673759E-2</v>
+        <v>3.6060234634483226E-2</v>
       </c>
       <c r="M28" s="10" t="str">
         <v>Actual/360</v>
@@ -5828,7 +5828,7 @@
         <v>10000</v>
       </c>
       <c r="P28" s="15">
-        <v>78.843110589166258</v>
+        <v>92.153932954790463</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
@@ -5851,10 +5851,10 @@
         <v>48249</v>
       </c>
       <c r="K29" s="9">
-        <v>3.0830190604218544E-2</v>
+        <v>3.6477850067591078E-2</v>
       </c>
       <c r="L29" s="9">
-        <v>3.0920531884376139E-2</v>
+        <v>3.6456269391778623E-2</v>
       </c>
       <c r="M29" s="10" t="str">
         <v>Actual/360</v>
@@ -5866,7 +5866,7 @@
         <v>10000</v>
       </c>
       <c r="P29" s="15">
-        <v>79.019137037850129</v>
+        <v>93.166021778989801</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
@@ -5889,10 +5889,10 @@
         <v>48339</v>
       </c>
       <c r="K30" s="9">
-        <v>3.0879635731970723E-2</v>
+        <v>3.6837157192763925E-2</v>
       </c>
       <c r="L30" s="9">
-        <v>3.0974131430625107E-2</v>
+        <v>3.6827484174562386E-2</v>
       </c>
       <c r="M30" s="10" t="str">
         <v>Actual/360</v>
@@ -5904,7 +5904,7 @@
         <v>10000</v>
       </c>
       <c r="P30" s="15">
-        <v>77.435328576562767</v>
+        <v>92.068710436405965</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
@@ -5927,10 +5927,10 @@
         <v>48431</v>
       </c>
       <c r="K31" s="9">
-        <v>3.0918311348839822E-2</v>
+        <v>3.7187684586195147E-2</v>
       </c>
       <c r="L31" s="9">
-        <v>3.1021173661076405E-2</v>
+        <v>3.7189447149281067E-2</v>
       </c>
       <c r="M31" s="10" t="str">
         <v>Actual/360</v>
@@ -5942,7 +5942,7 @@
         <v>10000</v>
       </c>
       <c r="P31" s="15">
-        <v>79.276332689417472</v>
+        <v>95.039698270384946</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
@@ -5965,10 +5965,10 @@
         <v>48523</v>
       </c>
       <c r="K32" s="9">
-        <v>3.094498824960823E-2</v>
+        <v>3.7521263372628511E-2</v>
       </c>
       <c r="L32" s="9">
-        <v>3.105404055261694E-2</v>
+        <v>3.753463754540385E-2</v>
       </c>
       <c r="M32" s="10" t="str">
         <v>Actual/360</v>
@@ -5980,7 +5980,7 @@
         <v>10000</v>
       </c>
       <c r="P32" s="15">
-        <v>79.360325856687723</v>
+        <v>95.921851504920937</v>
       </c>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.25">
@@ -6003,10 +6003,10 @@
         <v>48617</v>
       </c>
       <c r="K33" s="9">
-        <v>3.0962422180094151E-2</v>
+        <v>3.7845219160423937E-2</v>
       </c>
       <c r="L33" s="9">
-        <v>3.1077627406543518E-2</v>
+        <v>3.7870158523111271E-2</v>
       </c>
       <c r="M33" s="10" t="str">
         <v>Actual/360</v>
@@ -6018,7 +6018,7 @@
         <v>10000</v>
       </c>
       <c r="P33" s="15">
-        <v>81.147138228196965</v>
+        <v>98.883191699234985</v>
       </c>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
@@ -6041,10 +6041,10 @@
         <v>48704</v>
       </c>
       <c r="K34" s="9">
-        <v>3.0962447771356594E-2</v>
+        <v>3.8128070044578521E-2</v>
       </c>
       <c r="L34" s="9">
-        <v>3.1076843823253108E-2</v>
+        <v>3.8162117850993688E-2</v>
       </c>
       <c r="M34" s="10" t="str">
         <v>Actual/360</v>
@@ -6056,7 +6056,7 @@
         <v>10000</v>
       </c>
       <c r="P34" s="15">
-        <v>75.102372572861668</v>
+        <v>92.225118139901411</v>
       </c>
     </row>
     <row r="35" spans="2:16" x14ac:dyDescent="0.25">
@@ -6079,10 +6079,10 @@
         <v>48796</v>
       </c>
       <c r="K35" s="9">
-        <v>3.0954263489304523E-2</v>
+        <v>3.8415890571430467E-2</v>
       </c>
       <c r="L35" s="9">
-        <v>3.1080560136156538E-2</v>
+        <v>3.845945248468273E-2</v>
       </c>
       <c r="M35" s="10" t="str">
         <v>Actual/360</v>
@@ -6094,7 +6094,7 @@
         <v>10000</v>
       </c>
       <c r="P35" s="15">
-        <v>79.428098125733371</v>
+        <v>98.285267460855863</v>
       </c>
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.25">
@@ -6117,10 +6117,10 @@
         <v>48890</v>
       </c>
       <c r="K36" s="9">
-        <v>3.0939561611509347E-2</v>
+        <v>3.8712728997829515E-2</v>
       </c>
       <c r="L36" s="9">
-        <v>3.1070160375841677E-2</v>
+        <v>3.8757886446456752E-2</v>
       </c>
       <c r="M36" s="10" t="str">
         <v>Actual/360</v>
@@ -6132,7 +6132,7 @@
         <v>10000</v>
       </c>
       <c r="P36" s="15">
-        <v>81.12764098136438</v>
+        <v>101.20114794352597</v>
       </c>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.25">
@@ -6155,10 +6155,10 @@
         <v>48981</v>
       </c>
       <c r="K37" s="9">
-        <v>3.0913889881354351E-2</v>
+        <v>3.900184821157282E-2</v>
       </c>
       <c r="L37" s="9">
-        <v>3.1044205652901887E-2</v>
+        <v>3.9046984917428244E-2</v>
       </c>
       <c r="M37" s="10" t="str">
         <v>Actual/360</v>
@@ -6170,7 +6170,7 @@
         <v>10000</v>
       </c>
       <c r="P37" s="15">
-        <v>78.472853178168663</v>
+        <v>98.702100763499175</v>
       </c>
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.25">
@@ -6193,10 +6193,10 @@
         <v>49069</v>
       </c>
       <c r="K38" s="9">
-        <v>3.0877827647248779E-2</v>
+        <v>3.928288658289425E-2</v>
       </c>
       <c r="L38" s="9">
-        <v>3.1010466673227741E-2</v>
+        <v>3.932896560667451E-2</v>
       </c>
       <c r="M38" s="10" t="str">
         <v>Actual/360</v>
@@ -6208,7 +6208,7 @@
         <v>10000</v>
       </c>
       <c r="P38" s="15">
-        <v>75.80336297900115</v>
+        <v>96.137471482982136</v>
       </c>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.25">
@@ -6231,10 +6231,10 @@
         <v>49163</v>
       </c>
       <c r="K39" s="9">
-        <v>3.0836783702072879E-2</v>
+        <v>3.9588027123116376E-2</v>
       </c>
       <c r="L39" s="9">
-        <v>3.0979558913190253E-2</v>
+        <v>3.9637846345461018E-2</v>
       </c>
       <c r="M39" s="10" t="str">
         <v>Actual/360</v>
@@ -6246,7 +6246,7 @@
         <v>10000</v>
       </c>
       <c r="P39" s="15">
-        <v>80.891070495552327</v>
+        <v>103.49882101314822</v>
       </c>
     </row>
     <row r="40" spans="2:16" x14ac:dyDescent="0.25">
@@ -6269,10 +6269,10 @@
         <v>49254</v>
       </c>
       <c r="K40" s="9">
-        <v>3.0785349269493167E-2</v>
+        <v>3.9885086859658969E-2</v>
       </c>
       <c r="L40" s="9">
-        <v>3.0927242589718115E-2</v>
+        <v>3.9934871928259369E-2</v>
       </c>
       <c r="M40" s="10" t="str">
         <v>Actual/360</v>
@@ -6284,7 +6284,7 @@
         <v>10000</v>
       </c>
       <c r="P40" s="15">
-        <v>78.177196546231897</v>
+        <v>100.94648181865563</v>
       </c>
     </row>
     <row r="41" spans="2:16" x14ac:dyDescent="0.25">
@@ -6307,10 +6307,10 @@
         <v>49345</v>
       </c>
       <c r="K41" s="9">
-        <v>3.0725327289040649E-2</v>
+        <v>4.018479347622339E-2</v>
       </c>
       <c r="L41" s="9">
-        <v>3.087095089247964E-2</v>
+        <v>4.023622243720601E-2</v>
       </c>
       <c r="M41" s="10" t="str">
         <v>Actual/360</v>
@@ -6322,7 +6322,7 @@
         <v>10000</v>
       </c>
       <c r="P41" s="15">
-        <v>78.03490364487908</v>
+        <v>101.70822893849297</v>
       </c>
     </row>
     <row r="42" spans="2:16" x14ac:dyDescent="0.25">
@@ -6340,10 +6340,10 @@
         <v>49436</v>
       </c>
       <c r="K42" s="9">
-        <v>3.065671777363832E-2</v>
+        <v>4.0487146992607137E-2</v>
       </c>
       <c r="L42" s="9">
-        <v>3.0806007754347373E-2</v>
+        <v>4.0540268037977084E-2</v>
       </c>
       <c r="M42" s="10" t="str">
         <v>Actual/360</v>
@@ -6355,7 +6355,7 @@
         <v>10000</v>
       </c>
       <c r="P42" s="15">
-        <v>77.870741823489183</v>
+        <v>102.47678865155319</v>
       </c>
     </row>
     <row r="43" spans="2:16" x14ac:dyDescent="0.25">
@@ -6373,10 +6373,10 @@
         <v>49527</v>
       </c>
       <c r="K43" s="9">
-        <v>3.0579520737914478E-2</v>
+        <v>4.0792147428794223E-2</v>
       </c>
       <c r="L43" s="9">
-        <v>3.073241359812157E-2</v>
+        <v>4.0847009342245069E-2</v>
       </c>
       <c r="M43" s="10" t="str">
         <v>Actual/360</v>
@@ -6388,7 +6388,7 @@
         <v>10000</v>
       </c>
       <c r="P43" s="15">
-        <v>77.6847121508073</v>
+        <v>103.25216250400837</v>
       </c>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.25">
@@ -6406,10 +6406,10 @@
         <v>49618</v>
       </c>
       <c r="K44" s="9">
-        <v>3.0493736198549115E-2</v>
+        <v>4.1099794804981826E-2</v>
       </c>
       <c r="L44" s="9">
-        <v>3.0650168902917004E-2</v>
+        <v>4.1156446967137411E-2</v>
       </c>
       <c r="M44" s="10" t="str">
         <v>Actual/360</v>
@@ -6421,7 +6421,7 @@
         <v>10000</v>
       </c>
       <c r="P44" s="15">
-        <v>77.476815837929095</v>
+        <v>104.03435205581957</v>
       </c>
     </row>
     <row r="45" spans="2:16" x14ac:dyDescent="0.25">
@@ -6439,10 +6439,10 @@
         <v>49710</v>
       </c>
       <c r="K45" s="9">
-        <v>3.0394627691201492E-2</v>
+        <v>4.1412174434451998E-2</v>
       </c>
       <c r="L45" s="9">
-        <v>3.0560036628423444E-2</v>
+        <v>4.1472686852860277E-2</v>
       </c>
       <c r="M45" s="10" t="str">
         <v>Actual/360</v>
@@ -6454,7 +6454,7 @@
         <v>10000</v>
       </c>
       <c r="P45" s="15">
-        <v>78.097871383748796</v>
+        <v>105.98575529064293</v>
       </c>
     </row>
     <row r="46" spans="2:16" x14ac:dyDescent="0.25">
@@ -6472,10 +6472,10 @@
         <v>49800</v>
       </c>
       <c r="K46" s="9">
-        <v>3.0296404684273526E-2</v>
+        <v>4.1723030458893362E-2</v>
       </c>
       <c r="L46" s="9">
-        <v>3.0457881909207174E-2</v>
+        <v>4.1782732127829014E-2</v>
       </c>
       <c r="M46" s="10" t="str">
         <v>Actual/360</v>
@@ -6487,7 +6487,7 @@
         <v>10000</v>
       </c>
       <c r="P46" s="15">
-        <v>76.144704773017935</v>
+        <v>104.45683031957253</v>
       </c>
     </row>
     <row r="47" spans="2:16" x14ac:dyDescent="0.25">
@@ -6680,7 +6680,7 @@
         <v>122</v>
       </c>
       <c r="C6" s="31" t="str" cm="1">
-        <f t="array" ref="C6">_xll.qlDiscountingSwapEngine(C4)</f>
+        <f t="array" ref="C6">_xll.qlDiscountingSwapEngine(C4,FALSE)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R6C3DiscountingSwapEngine,A</v>
       </c>
       <c r="E6" s="98" t="s">
@@ -6946,12 +6946,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C8Schedule,A</v>
       </c>
       <c r="I17" s="26" t="str" cm="1">
-        <f t="array" ref="I17">_xll.qlOvernightIndexedSwap("Payer",$C$21,H17,$C$22,"Act/360",$C$19)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C9OvernightIndexedSwap,A</v>
+        <f t="array" ref="I17">_xll.qlOvernightIndexedSwap("Payer",$C$21,H17,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C9OvernightIndexedSwap,G</v>
       </c>
       <c r="J17" s="109" cm="1">
         <f t="array" ref="J17">_xll.qlSwapLegBPS(I17,1,_xll.qlInstrumentSetPricingEngine(I17,$C$6))*10000</f>
-        <v>77005.886415961038</v>
+        <v>75803.2600393584</v>
       </c>
       <c r="K17" s="26" t="str" cm="1">
         <f t="array" ref="K17">_xll.qlEuropeanExercise(F17,$C$2)</f>
@@ -6963,22 +6963,22 @@
       </c>
       <c r="M17" s="88" cm="1">
         <f t="array" ref="M17">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$7))</f>
-        <v>219.69689498119271</v>
+        <v>480.19741230417134</v>
       </c>
       <c r="N17" s="109" cm="1">
         <f t="array" ref="N17">_xll.qlSwaptionAnnuity(L17,M17)</f>
-        <v>77005.886415961038</v>
+        <v>75803.2600393584</v>
       </c>
       <c r="O17" s="28" cm="1">
         <f t="array" ref="O17">_xll.qlSwaptionImpliedVolatility(L17,M17,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8192074375075778E-3</v>
+        <v>6.819207895275751E-3</v>
       </c>
       <c r="Q17" s="28" cm="1">
         <f t="array" ref="Q17">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F17,S17,$C$22)</f>
         <v>6.8192074362781394E-3</v>
       </c>
       <c r="R17" s="112">
-        <f t="shared" ref="R17:R25" si="0">G17-F17</f>
+        <f>G17-F17</f>
         <v>2</v>
       </c>
       <c r="S17" s="113" t="str">
@@ -6993,7 +6993,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V17" s="114">
-        <f t="shared" ref="V17:V26" si="1">$C$30</f>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W17" s="115" t="b" cm="1">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="X17" s="28" cm="1">
         <f t="array" ref="X17:X26">_xll.qlGsrVolatility(C31,C43)</f>
-        <v>7.2053033222295561E-3</v>
+        <v>7.2562982901529325E-3</v>
       </c>
     </row>
     <row r="18" spans="2:24" x14ac:dyDescent="0.25">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="C18" s="52" t="str">
         <f>'Sofr swap'!C14</f>
-        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R14C3,B</v>
+        <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R14C3,A</v>
       </c>
       <c r="E18" s="98" t="s">
         <v>98</v>
@@ -7029,12 +7029,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C8Schedule,A</v>
       </c>
       <c r="I18" s="31" t="str" cm="1">
-        <f t="array" ref="I18">_xll.qlOvernightIndexedSwap("Payer",$C$21,H18,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I18">_xll.qlOvernightIndexedSwap("Payer",$C$21,H18,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J18" s="110" cm="1">
         <f t="array" ref="J18">_xll.qlSwapLegBPS(I18,1,_xll.qlInstrumentSetPricingEngine(I18,$C$6))*10000</f>
-        <v>67347.703367765615</v>
+        <v>66149.320380348523</v>
       </c>
       <c r="K18" s="31" t="str" cm="1">
         <f t="array" ref="K18">_xll.qlEuropeanExercise(F18,$C$2)</f>
@@ -7046,26 +7046,26 @@
       </c>
       <c r="M18" s="90" cm="1">
         <f t="array" ref="M18">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$7))</f>
-        <v>274.7466576732611</v>
+        <v>514.76204370168534</v>
       </c>
       <c r="N18" s="110" cm="1">
         <f t="array" ref="N18">_xll.qlSwaptionAnnuity(L18,M18)</f>
-        <v>67347.703367765615</v>
+        <v>66149.320380348523</v>
       </c>
       <c r="O18" s="33" cm="1">
         <f t="array" ref="O18">_xll.qlSwaptionImpliedVolatility(L18,M18,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8439003522771788E-3</v>
+        <v>6.8439003670021578E-3</v>
       </c>
       <c r="Q18" s="33" cm="1">
         <f t="array" ref="Q18">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F18,S18,$C$22)</f>
         <v>6.8439003518695187E-3</v>
       </c>
       <c r="R18" s="116">
-        <f t="shared" si="0"/>
+        <f>G18-F18</f>
         <v>2</v>
       </c>
       <c r="S18" s="117" t="str">
-        <f t="shared" ref="S18:S25" si="2">ROUND(($C$17-G18)/365.25,0)&amp;"y"</f>
+        <f>ROUND(($C$17-G18)/365.25,0)&amp;"y"</f>
         <v>8y</v>
       </c>
       <c r="T18" s="31" t="str" cm="1">
@@ -7076,7 +7076,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V18" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W18" s="63" t="b" cm="1">
@@ -7084,7 +7084,7 @@
         <v>1</v>
       </c>
       <c r="X18" s="33">
-        <v>7.2590401039309077E-3</v>
+        <v>7.2854447762798731E-3</v>
       </c>
     </row>
     <row r="19" spans="2:24" x14ac:dyDescent="0.25">
@@ -7111,12 +7111,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C8Schedule,A</v>
       </c>
       <c r="I19" s="31" t="str" cm="1">
-        <f t="array" ref="I19">_xll.qlOvernightIndexedSwap("Payer",$C$21,H19,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I19">_xll.qlOvernightIndexedSwap("Payer",$C$21,H19,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J19" s="110" cm="1">
         <f t="array" ref="J19">_xll.qlSwapLegBPS(I19,1,_xll.qlInstrumentSetPricingEngine(I19,$C$6))*10000</f>
-        <v>57947.189586901935</v>
+        <v>56766.422970738095</v>
       </c>
       <c r="K19" s="31" t="str" cm="1">
         <f t="array" ref="K19">_xll.qlEuropeanExercise(F19,$C$2)</f>
@@ -7128,26 +7128,26 @@
       </c>
       <c r="M19" s="90" cm="1">
         <f t="array" ref="M19">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$7))</f>
-        <v>293.68786762058801</v>
+        <v>519.2238834625033</v>
       </c>
       <c r="N19" s="110" cm="1">
         <f t="array" ref="N19">_xll.qlSwaptionAnnuity(L19,M19)</f>
-        <v>57947.189586901935</v>
+        <v>56766.422970738087</v>
       </c>
       <c r="O19" s="33" cm="1">
         <f t="array" ref="O19">_xll.qlSwaptionImpliedVolatility(L19,M19,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8685932680086449E-3</v>
+        <v>6.8685932718781911E-3</v>
       </c>
       <c r="Q19" s="33" cm="1">
         <f t="array" ref="Q19">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F19,S19,$C$22)</f>
         <v>6.8685932674608981E-3</v>
       </c>
       <c r="R19" s="116">
-        <f t="shared" si="0"/>
+        <f>G19-F19</f>
         <v>4</v>
       </c>
       <c r="S19" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G19)/365.25,0)&amp;"y"</f>
         <v>7y</v>
       </c>
       <c r="T19" s="31" t="str" cm="1">
@@ -7158,7 +7158,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V19" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W19" s="63" t="b" cm="1">
@@ -7166,7 +7166,7 @@
         <v>1</v>
       </c>
       <c r="X19" s="33">
-        <v>7.3091903500280171E-3</v>
+        <v>7.3317640293017773E-3</v>
       </c>
     </row>
     <row r="20" spans="2:24" x14ac:dyDescent="0.25">
@@ -7186,12 +7186,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C8Schedule,A</v>
       </c>
       <c r="I20" s="31" t="str" cm="1">
-        <f t="array" ref="I20">_xll.qlOvernightIndexedSwap("Payer",$C$21,H20,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I20">_xll.qlOvernightIndexedSwap("Payer",$C$21,H20,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J20" s="110" cm="1">
         <f t="array" ref="J20">_xll.qlSwapLegBPS(I20,1,_xll.qlInstrumentSetPricingEngine(I20,$C$6))*10000</f>
-        <v>48901.706248573246</v>
+        <v>47759.243446805121</v>
       </c>
       <c r="K20" s="31" t="str" cm="1">
         <f t="array" ref="K20">_xll.qlEuropeanExercise(F20,$C$2)</f>
@@ -7203,26 +7203,26 @@
       </c>
       <c r="M20" s="90" cm="1">
         <f t="array" ref="M20">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$7))</f>
-        <v>286.54787185933537</v>
+        <v>493.61995406800253</v>
       </c>
       <c r="N20" s="110" cm="1">
         <f t="array" ref="N20">_xll.qlSwaptionAnnuity(L20,M20)</f>
-        <v>48901.706248573246</v>
+        <v>47759.243446805121</v>
       </c>
       <c r="O20" s="33" cm="1">
         <f t="array" ref="O20">_xll.qlSwaptionImpliedVolatility(L20,M20,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8710196103278567E-3</v>
+        <v>6.8710196122747777E-3</v>
       </c>
       <c r="Q20" s="33" cm="1">
         <f t="array" ref="Q20">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F20,S20,$C$22)</f>
         <v>6.8710196098611381E-3</v>
       </c>
       <c r="R20" s="116">
-        <f t="shared" si="0"/>
+        <f>G20-F20</f>
         <v>4</v>
       </c>
       <c r="S20" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G20)/365.25,0)&amp;"y"</f>
         <v>6y</v>
       </c>
       <c r="T20" s="31" t="str" cm="1">
@@ -7233,7 +7233,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V20" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W20" s="63" t="b" cm="1">
@@ -7241,7 +7241,7 @@
         <v>1</v>
       </c>
       <c r="X20" s="33">
-        <v>7.2420658823182148E-3</v>
+        <v>7.2499818707807877E-3</v>
       </c>
     </row>
     <row r="21" spans="2:24" x14ac:dyDescent="0.25">
@@ -7267,12 +7267,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C8Schedule,A</v>
       </c>
       <c r="I21" s="31" t="str" cm="1">
-        <f t="array" ref="I21">_xll.qlOvernightIndexedSwap("Payer",$C$21,H21,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I21">_xll.qlOvernightIndexedSwap("Payer",$C$21,H21,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J21" s="110" cm="1">
         <f t="array" ref="J21">_xll.qlSwapLegBPS(I21,1,_xll.qlInstrumentSetPricingEngine(I21,$C$6))*10000</f>
-        <v>40129.589162277225</v>
+        <v>39055.847564585856</v>
       </c>
       <c r="K21" s="31" t="str" cm="1">
         <f t="array" ref="K21">_xll.qlEuropeanExercise(F21,$C$2)</f>
@@ -7284,26 +7284,26 @@
       </c>
       <c r="M21" s="90" cm="1">
         <f t="array" ref="M21">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$7))</f>
-        <v>261.31005037414184</v>
+        <v>445.14555434793988</v>
       </c>
       <c r="N21" s="110" cm="1">
         <f t="array" ref="N21">_xll.qlSwaptionAnnuity(L21,M21)</f>
-        <v>40129.589162277225</v>
+        <v>39055.847564585856</v>
       </c>
       <c r="O21" s="33" cm="1">
         <f t="array" ref="O21">_xll.qlSwaptionImpliedVolatility(L21,M21,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8386420679046305E-3</v>
+        <v>6.8386420695241458E-3</v>
       </c>
       <c r="Q21" s="33" cm="1">
         <f t="array" ref="Q21">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F21,S21,$C$22)</f>
         <v>6.8386420675278876E-3</v>
       </c>
       <c r="R21" s="116">
-        <f t="shared" si="0"/>
+        <f>G21-F21</f>
         <v>4</v>
       </c>
       <c r="S21" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G21)/365.25,0)&amp;"y"</f>
         <v>5y</v>
       </c>
       <c r="T21" s="31" t="str" cm="1">
@@ -7314,7 +7314,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V21" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W21" s="63" t="b" cm="1">
@@ -7322,7 +7322,7 @@
         <v>1</v>
       </c>
       <c r="X21" s="33">
-        <v>7.1126731090583378E-3</v>
+        <v>7.0519393916380711E-3</v>
       </c>
     </row>
     <row r="22" spans="2:24" x14ac:dyDescent="0.25">
@@ -7348,12 +7348,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C8Schedule,A</v>
       </c>
       <c r="I22" s="31" t="str" cm="1">
-        <f t="array" ref="I22">_xll.qlOvernightIndexedSwap("Payer",$C$21,H22,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I22">_xll.qlOvernightIndexedSwap("Payer",$C$21,H22,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J22" s="110" cm="1">
         <f t="array" ref="J22">_xll.qlSwapLegBPS(I22,1,_xll.qlInstrumentSetPricingEngine(I22,$C$6))*10000</f>
-        <v>31579.295736941924</v>
+        <v>30614.041334853744</v>
       </c>
       <c r="K22" s="31" t="str" cm="1">
         <f t="array" ref="K22">_xll.qlEuropeanExercise(F22,$C$2)</f>
@@ -7365,26 +7365,26 @@
       </c>
       <c r="M22" s="90" cm="1">
         <f t="array" ref="M22">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$7))</f>
-        <v>223.48777131172506</v>
+        <v>378.67641020372002</v>
       </c>
       <c r="N22" s="110" cm="1">
         <f t="array" ref="N22">_xll.qlSwaptionAnnuity(L22,M22)</f>
-        <v>31579.295736941924</v>
+        <v>30614.04133485374</v>
       </c>
       <c r="O22" s="33" cm="1">
         <f t="array" ref="O22">_xll.qlSwaptionImpliedVolatility(L22,M22,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8094752903852052E-3</v>
+        <v>6.8094752919335361E-3</v>
       </c>
       <c r="Q22" s="33" cm="1">
         <f t="array" ref="Q22">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F22,S22,$C$22)</f>
         <v>6.8094752901471274E-3</v>
       </c>
       <c r="R22" s="116">
-        <f t="shared" si="0"/>
+        <f>G22-F22</f>
         <v>2</v>
       </c>
       <c r="S22" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G22)/365.25,0)&amp;"y"</f>
         <v>4y</v>
       </c>
       <c r="T22" s="31" t="str" cm="1">
@@ -7395,7 +7395,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V22" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W22" s="63" t="b" cm="1">
@@ -7403,7 +7403,7 @@
         <v>1</v>
       </c>
       <c r="X22" s="33">
-        <v>7.0384062876536115E-3</v>
+        <v>7.0789799045768848E-3</v>
       </c>
     </row>
     <row r="23" spans="2:24" x14ac:dyDescent="0.25">
@@ -7423,12 +7423,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C8Schedule,A</v>
       </c>
       <c r="I23" s="31" t="str" cm="1">
-        <f t="array" ref="I23">_xll.qlOvernightIndexedSwap("Payer",$C$21,H23,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I23">_xll.qlOvernightIndexedSwap("Payer",$C$21,H23,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J23" s="110" cm="1">
         <f t="array" ref="J23">_xll.qlSwapLegBPS(I23,1,_xll.qlInstrumentSetPricingEngine(I23,$C$6))*10000</f>
-        <v>23315.518591450636</v>
+        <v>22505.50178121102</v>
       </c>
       <c r="K23" s="31" t="str" cm="1">
         <f t="array" ref="K23">_xll.qlEuropeanExercise(F23,$C$2)</f>
@@ -7440,26 +7440,26 @@
       </c>
       <c r="M23" s="90" cm="1">
         <f t="array" ref="M23">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$7))</f>
-        <v>176.37308441929778</v>
+        <v>298.39887641285605</v>
       </c>
       <c r="N23" s="110" cm="1">
         <f t="array" ref="N23">_xll.qlSwaptionAnnuity(L23,M23)</f>
-        <v>23315.518591450636</v>
+        <v>22505.501781211016</v>
       </c>
       <c r="O23" s="33" cm="1">
         <f t="array" ref="O23">_xll.qlSwaptionImpliedVolatility(L23,M23,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.789977576566685E-3</v>
+        <v>6.7899775780790048E-3</v>
       </c>
       <c r="Q23" s="33" cm="1">
         <f t="array" ref="Q23">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F23,S23,$C$22)</f>
         <v>6.7899775764584816E-3</v>
       </c>
       <c r="R23" s="116">
-        <f t="shared" si="0"/>
+        <f>G23-F23</f>
         <v>2</v>
       </c>
       <c r="S23" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G23)/365.25,0)&amp;"y"</f>
         <v>3y</v>
       </c>
       <c r="T23" s="31" t="str" cm="1">
@@ -7470,7 +7470,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V23" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W23" s="63" t="b" cm="1">
@@ -7478,7 +7478,7 @@
         <v>1</v>
       </c>
       <c r="X23" s="33">
-        <v>7.0763069751538362E-3</v>
+        <v>6.9660793842538805E-3</v>
       </c>
     </row>
     <row r="24" spans="2:24" x14ac:dyDescent="0.25">
@@ -7498,12 +7498,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C8Schedule,A</v>
       </c>
       <c r="I24" s="31" t="str" cm="1">
-        <f t="array" ref="I24">_xll.qlOvernightIndexedSwap("Payer",$C$21,H24,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I24">_xll.qlOvernightIndexedSwap("Payer",$C$21,H24,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J24" s="110" cm="1">
         <f t="array" ref="J24">_xll.qlSwapLegBPS(I24,1,_xll.qlInstrumentSetPricingEngine(I24,$C$6))*10000</f>
-        <v>15306.987939780221</v>
+        <v>14705.474136934443</v>
       </c>
       <c r="K24" s="31" t="str" cm="1">
         <f t="array" ref="K24">_xll.qlEuropeanExercise(F24,$C$2)</f>
@@ -7515,26 +7515,26 @@
       </c>
       <c r="M24" s="90" cm="1">
         <f t="array" ref="M24">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$7))</f>
-        <v>123.96499712474312</v>
+        <v>208.87169946565118</v>
       </c>
       <c r="N24" s="110" cm="1">
         <f t="array" ref="N24">_xll.qlSwaptionAnnuity(L24,M24)</f>
-        <v>15306.98793978022</v>
+        <v>14705.474136934441</v>
       </c>
       <c r="O24" s="33" cm="1">
         <f t="array" ref="O24">_xll.qlSwaptionImpliedVolatility(L24,M24,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.8705740177160265E-3</v>
+        <v>6.8707896854334058E-3</v>
       </c>
       <c r="Q24" s="33" cm="1">
         <f t="array" ref="Q24">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F24,S24,$C$22)</f>
         <v>6.8705740176875649E-3</v>
       </c>
       <c r="R24" s="116">
-        <f t="shared" si="0"/>
+        <f>G24-F24</f>
         <v>2</v>
       </c>
       <c r="S24" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G24)/365.25,0)&amp;"y"</f>
         <v>2y</v>
       </c>
       <c r="T24" s="31" t="str" cm="1">
@@ -7545,7 +7545,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V24" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W24" s="63" t="b" cm="1">
@@ -7553,7 +7553,7 @@
         <v>1</v>
       </c>
       <c r="X24" s="33">
-        <v>7.7774538867825E-3</v>
+        <v>7.8011054462023364E-3</v>
       </c>
     </row>
     <row r="25" spans="2:24" x14ac:dyDescent="0.25">
@@ -7573,12 +7573,12 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C8Schedule,A</v>
       </c>
       <c r="I25" s="36" t="str" cm="1">
-        <f t="array" ref="I25">_xll.qlOvernightIndexedSwap("Payer",$C$21,H25,$C$22,"Act/360",$C$19)</f>
+        <f t="array" ref="I25">_xll.qlOvernightIndexedSwap("Payer",$C$21,H25,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C9OvernightIndexedSwap,A</v>
       </c>
       <c r="J25" s="111" cm="1">
         <f t="array" ref="J25">_xll.qlSwapLegBPS(I25,1,_xll.qlInstrumentSetPricingEngine(I25,$C$6))*10000</f>
-        <v>7503.3224394089848</v>
+        <v>7171.0842364683413</v>
       </c>
       <c r="K25" s="36" t="str" cm="1">
         <f t="array" ref="K25">_xll.qlEuropeanExercise(F25,$C$2)</f>
@@ -7590,26 +7590,26 @@
       </c>
       <c r="M25" s="92" cm="1">
         <f t="array" ref="M25">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$7))</f>
-        <v>63.005644741445415</v>
+        <v>107.37919557367384</v>
       </c>
       <c r="N25" s="111" cm="1">
         <f t="array" ref="N25">_xll.qlSwaptionAnnuity(L25,M25)</f>
-        <v>7503.3224394089848</v>
+        <v>7171.0842364683413</v>
       </c>
       <c r="O25" s="38" cm="1">
         <f t="array" ref="O25">_xll.qlSwaptionImpliedVolatility(L25,M25,$C$4,0.01,,,,,"Normal")</f>
-        <v>6.7898728295228339E-3</v>
+        <v>6.789872830937918E-3</v>
       </c>
       <c r="Q25" s="33" cm="1">
         <f t="array" ref="Q25">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F25,S25,$C$22)</f>
         <v>6.7898728295167242E-3</v>
       </c>
       <c r="R25" s="116">
-        <f t="shared" si="0"/>
+        <f>G25-F25</f>
         <v>4</v>
       </c>
       <c r="S25" s="117" t="str">
-        <f t="shared" si="2"/>
+        <f>ROUND(($C$17-G25)/365.25,0)&amp;"y"</f>
         <v>1y</v>
       </c>
       <c r="T25" s="31" t="str" cm="1">
@@ -7620,7 +7620,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V25" s="118">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W25" s="63" t="b" cm="1">
@@ -7628,7 +7628,7 @@
         <v>1</v>
       </c>
       <c r="X25" s="33">
-        <v>6.5434227807583279E-3</v>
+        <v>6.4311298987523163E-3</v>
       </c>
     </row>
     <row r="26" spans="2:24" x14ac:dyDescent="0.25">
@@ -7640,7 +7640,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V26" s="120">
-        <f t="shared" si="1"/>
+        <f>$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W26" s="39"/>
@@ -7667,7 +7667,7 @@
       </c>
       <c r="C31" s="31" t="str" cm="1">
         <f t="array" ref="C31">_xll.qlGsr(C4,F17:F25,U17:U26,V17:V26,,M17:M25)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R31C3Gsr,A</v>
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R31C3Gsr,B</v>
       </c>
     </row>
     <row r="32" spans="2:24" x14ac:dyDescent="0.25">
@@ -7676,7 +7676,7 @@
       </c>
       <c r="C32" s="31" t="str" cm="1">
         <f t="array" ref="C32">_xll.qlGaussian1dJamshidianSwaptionEngine(C31)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R32C3Gaussian1dJamshidianSwaptionEngine,A</v>
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R32C3Gaussian1dJamshidianSwaptionEngine,B</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="C33" s="36" t="str" cm="1">
         <f t="array" ref="C33">_xll.qlGaussian1dSwaptionEngine(C31)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R33C3Gaussian1dSwaptionEngine,A</v>
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R33C3Gaussian1dSwaptionEngine,B</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
@@ -7796,128 +7796,128 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" s="87" t="str">
-        <f t="shared" ref="B53:B61" si="3">E17&amp;"-"&amp;S17</f>
+        <f>E17&amp;"-"&amp;S17</f>
         <v>1y-9y</v>
       </c>
       <c r="C53" s="88" cm="1">
         <f t="array" ref="C53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$32,$C$43))</f>
-        <v>219.68823932629044</v>
+        <v>480.19295857890654</v>
       </c>
       <c r="D53" s="88" cm="1">
         <f t="array" ref="D53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$33,$C$43))</f>
-        <v>212.72632926709488</v>
+        <v>477.74924495888234</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B54" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E18&amp;"-"&amp;S18</f>
         <v>2y-8y</v>
       </c>
       <c r="C54" s="90" cm="1">
         <f t="array" ref="C54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$32,$C$43))</f>
-        <v>274.7410382173785</v>
+        <v>514.75686806025317</v>
       </c>
       <c r="D54" s="90" cm="1">
         <f t="array" ref="D54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$33,$C$43))</f>
-        <v>269.40636210281366</v>
+        <v>513.50611040521835</v>
       </c>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B55" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E19&amp;"-"&amp;S19</f>
         <v>3y-7y</v>
       </c>
       <c r="C55" s="90" cm="1">
         <f t="array" ref="C55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$32,$C$43))</f>
-        <v>293.67828165531057</v>
+        <v>519.21992874969453</v>
       </c>
       <c r="D55" s="90" cm="1">
         <f t="array" ref="D55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$33,$C$43))</f>
-        <v>288.01669189572277</v>
+        <v>517.23545516948286</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B56" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E20&amp;"-"&amp;S20</f>
         <v>4y-6y</v>
       </c>
       <c r="C56" s="90" cm="1">
         <f t="array" ref="C56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$32,$C$43))</f>
-        <v>286.52597469989405</v>
+        <v>493.60804779991349</v>
       </c>
       <c r="D56" s="90" cm="1">
         <f t="array" ref="D56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$33,$C$43))</f>
-        <v>281.21373905552639</v>
+        <v>491.03774318071919</v>
       </c>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B57" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E21&amp;"-"&amp;S21</f>
         <v>5y-5y</v>
       </c>
       <c r="C57" s="90" cm="1">
         <f t="array" ref="C57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$32,$C$43))</f>
-        <v>261.28788564765193</v>
+        <v>445.12383139248038</v>
       </c>
       <c r="D57" s="90" cm="1">
         <f t="array" ref="D57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$33,$C$43))</f>
-        <v>256.6122551395386</v>
+        <v>442.42184610809704</v>
       </c>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B58" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E22&amp;"-"&amp;S22</f>
         <v>6y-4y</v>
       </c>
       <c r="C58" s="90" cm="1">
         <f t="array" ref="C58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$32,$C$43))</f>
-        <v>223.48333562325126</v>
+        <v>378.66930593822264</v>
       </c>
       <c r="D58" s="90" cm="1">
         <f t="array" ref="D58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$33,$C$43))</f>
-        <v>219.42220813138732</v>
+        <v>376.09095103371908</v>
       </c>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B59" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E23&amp;"-"&amp;S23</f>
         <v>7y-3y</v>
       </c>
       <c r="C59" s="90" cm="1">
         <f t="array" ref="C59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$32,$C$43))</f>
-        <v>176.36912411204591</v>
+        <v>298.39373179886041</v>
       </c>
       <c r="D59" s="90" cm="1">
         <f t="array" ref="D59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$33,$C$43))</f>
-        <v>173.22009056754075</v>
+        <v>296.23172499493859</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B60" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E24&amp;"-"&amp;S24</f>
         <v>8y-2y</v>
       </c>
       <c r="C60" s="90" cm="1">
         <f t="array" ref="C60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$32,$C$43))</f>
-        <v>123.96101111691891</v>
+        <v>208.86665999869419</v>
       </c>
       <c r="D60" s="90" cm="1">
         <f t="array" ref="D60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$33,$C$43))</f>
-        <v>121.73038636572213</v>
+        <v>207.31794600871279</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B61" s="89" t="str">
-        <f t="shared" si="3"/>
+        <f>E25&amp;"-"&amp;S25</f>
         <v>9y-1y</v>
       </c>
       <c r="C61" s="90" cm="1">
         <f t="array" ref="C61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$32,$C$43))</f>
-        <v>62.998974459548236</v>
+        <v>107.37144562488741</v>
       </c>
       <c r="D61" s="90" cm="1">
         <f t="array" ref="D61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$33,$C$43))</f>
-        <v>61.879872815595782</v>
+        <v>106.57878015619599</v>
       </c>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.25">
@@ -7927,7 +7927,7 @@
       <c r="C62" s="34"/>
       <c r="D62" s="92" cm="1">
         <f t="array" ref="D62">_xll.qlInstrumentNPV(C48,_xll.qlInstrumentSetPricingEngine(C48,$C$33,$C$43))</f>
-        <v>384.60558714558329</v>
+        <v>631.27448041042044</v>
       </c>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.25">
@@ -7937,7 +7937,7 @@
       <c r="C64" s="121"/>
       <c r="D64" s="122">
         <f>D62-MAX(D53:D61)</f>
-        <v>96.588895249860514</v>
+        <v>114.03902524093758</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix workbook test for QuantLib v1.43
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
+++ b/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989D1F3F-D783-4A3B-BEEB-8FB51FCDD782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1ECC03-BFAD-403D-B7EE-D449B933C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
+    <workbookView xWindow="14655" yWindow="-20355" windowWidth="22170" windowHeight="15285" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="174">
   <si>
     <t>Evaluation date</t>
   </si>
@@ -588,6 +588,9 @@
   </si>
   <si>
     <t>European swaptions and calibration helpers</t>
+  </si>
+  <si>
+    <t>Quote Currency Payment Frequency</t>
   </si>
 </sst>
 </file>
@@ -860,7 +863,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -951,7 +954,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1073,9 +1075,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Link" xfId="2" builtinId="8"/>
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1091,7 +1093,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1408,15 +1410,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6008FAD-AC53-4BA7-8BFE-AA0AF33C510B}">
   <dimension ref="B2:C25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="17"/>
-    <col min="2" max="2" width="16.7109375" style="17" customWidth="1"/>
-    <col min="3" max="3" width="62.140625" style="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.85546875" style="17"/>
+    <col min="1" max="1" width="8.88671875" style="17"/>
+    <col min="2" max="2" width="16.6640625" style="17" customWidth="1"/>
+    <col min="3" max="3" width="62.109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="17"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="16" t="s">
         <v>152</v>
       </c>
@@ -1424,7 +1426,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="16" t="s">
         <v>154</v>
       </c>
@@ -1432,7 +1434,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
         <v>156</v>
       </c>
@@ -1440,35 +1442,35 @@
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="16" t="s">
         <v>159</v>
       </c>
       <c r="C10" s="20" t="str" cm="1">
         <f t="array" ref="C10">_xll.qlVersion()</f>
-        <v>1.42.1</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="16" t="s">
         <v>160</v>
       </c>
       <c r="C11" s="20" t="str" cm="1">
         <f t="array" ref="C11">_xll.qlXlOilVersion()</f>
-        <v>0.42.2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+        <v>0.43.0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="19" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B14" s="20" t="str" cm="1">
         <f t="array" ref="B14:C15">_xll.xloVersion()</f>
         <v>Version</v>
@@ -1477,7 +1479,7 @@
         <v>0.22.1</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="20" t="str">
         <v>BuildDate</v>
       </c>
@@ -1485,12 +1487,12 @@
         <v>"May 10 2026"</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="19" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" s="17" t="s">
         <v>163</v>
       </c>
@@ -1498,7 +1500,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" s="17" t="s">
         <v>57</v>
       </c>
@@ -1506,7 +1508,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="17" t="s">
         <v>92</v>
       </c>
@@ -1514,7 +1516,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:3" ht="72" x14ac:dyDescent="0.3">
       <c r="B25" s="17" t="s">
         <v>167</v>
       </c>
@@ -1533,19 +1535,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8757F0-0B54-406F-8B83-8898C4C64D27}">
-  <dimension ref="B2:M88"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:M89"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1555,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
         <v>1</v>
       </c>
@@ -1562,7 +1564,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="24" t="s">
         <v>2</v>
       </c>
@@ -1571,7 +1573,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R5C3Estr,A</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>3</v>
       </c>
@@ -1580,7 +1582,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R6C3Euribor,A</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="34" t="s">
         <v>4</v>
       </c>
@@ -1589,7 +1591,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R7C3Sofr,A</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
@@ -1597,7 +1599,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="24" t="s">
         <v>21</v>
       </c>
@@ -1620,7 +1622,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>22</v>
       </c>
@@ -1646,7 +1648,7 @@
         <v>1.9608084420931857E-2</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B13" s="34" t="s">
         <v>23</v>
       </c>
@@ -1672,7 +1674,7 @@
         <v>1.9561814398052216E-2</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B14" s="44" t="s">
         <v>24</v>
       </c>
@@ -1699,7 +1701,7 @@
         <v>1.9508413197557743E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E15" s="29" t="s">
         <v>12</v>
       </c>
@@ -1719,7 +1721,7 @@
         <v>1.9423329540682495E-2</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E16" s="29" t="s">
         <v>13</v>
       </c>
@@ -1739,7 +1741,7 @@
         <v>1.9707419970420838E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E17" s="29" t="s">
         <v>14</v>
       </c>
@@ -1759,7 +1761,7 @@
         <v>2.0304501541429942E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E18" s="29" t="s">
         <v>15</v>
       </c>
@@ -1779,7 +1781,7 @@
         <v>2.1056614418825545E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E19" s="29" t="s">
         <v>16</v>
       </c>
@@ -1799,7 +1801,7 @@
         <v>2.1804311905509664E-2</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E20" s="29" t="s">
         <v>17</v>
       </c>
@@ -1819,7 +1821,7 @@
         <v>2.3305383398994673E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E21" s="29" t="s">
         <v>18</v>
       </c>
@@ -1839,7 +1841,7 @@
         <v>2.5394439430906784E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E22" s="34" t="s">
         <v>19</v>
       </c>
@@ -1859,7 +1861,7 @@
         <v>2.6618940661949898E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
         <v>28</v>
       </c>
@@ -1867,7 +1869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B27" s="24" t="s">
         <v>21</v>
       </c>
@@ -1890,7 +1892,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>22</v>
       </c>
@@ -1916,7 +1918,7 @@
         <v>2.1489715124367082E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B29" s="34" t="s">
         <v>23</v>
       </c>
@@ -1942,7 +1944,7 @@
         <v>2.1547204844790901E-2</v>
       </c>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B30" s="44" t="s">
         <v>24</v>
       </c>
@@ -1969,7 +1971,7 @@
         <v>2.1964582886470737E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E31" s="29" t="s">
         <v>14</v>
       </c>
@@ -1990,7 +1992,7 @@
         <v>2.2568918764418931E-2</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E32" s="29" t="s">
         <v>15</v>
       </c>
@@ -2010,7 +2012,7 @@
         <v>2.3294217587170939E-2</v>
       </c>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E33" s="29" t="s">
         <v>16</v>
       </c>
@@ -2030,7 +2032,7 @@
         <v>2.3957140103980739E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E34" s="29" t="s">
         <v>17</v>
       </c>
@@ -2050,7 +2052,7 @@
         <v>2.5305364889382738E-2</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E35" s="29" t="s">
         <v>18</v>
       </c>
@@ -2070,7 +2072,7 @@
         <v>2.7224289747691924E-2</v>
       </c>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E36" s="34" t="s">
         <v>19</v>
       </c>
@@ -2090,12 +2092,12 @@
         <v>2.8266282940571708E-2</v>
       </c>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
       <c r="F37" s="6"/>
       <c r="G37" s="4"/>
     </row>
-    <row r="38" spans="2:10" s="8" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B39" s="5" t="s">
         <v>29</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B41" s="24" t="s">
         <v>21</v>
       </c>
@@ -2126,7 +2128,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>22</v>
       </c>
@@ -2152,7 +2154,7 @@
         <v>3.7511961223903233E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B43" s="34" t="s">
         <v>23</v>
       </c>
@@ -2178,7 +2180,7 @@
         <v>3.6998167414587564E-2</v>
       </c>
     </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B44" s="44" t="s">
         <v>24</v>
       </c>
@@ -2205,7 +2207,7 @@
         <v>3.6350945887968909E-2</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E45" s="29" t="s">
         <v>12</v>
       </c>
@@ -2225,7 +2227,7 @@
         <v>3.4626290911888569E-2</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E46" s="29" t="s">
         <v>13</v>
       </c>
@@ -2245,7 +2247,7 @@
         <v>3.2751768392570955E-2</v>
       </c>
     </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E47" s="29" t="s">
         <v>14</v>
       </c>
@@ -2265,7 +2267,7 @@
         <v>3.2377367024610644E-2</v>
       </c>
     </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E48" s="29" t="s">
         <v>15</v>
       </c>
@@ -2285,7 +2287,7 @@
         <v>3.2661635352545959E-2</v>
       </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
       <c r="E49" s="29" t="s">
         <v>16</v>
       </c>
@@ -2305,7 +2307,7 @@
         <v>3.3148897734764607E-2</v>
       </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.3">
       <c r="E50" s="29" t="s">
         <v>17</v>
       </c>
@@ -2325,7 +2327,7 @@
         <v>3.4367701312975452E-2</v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
       <c r="E51" s="29" t="s">
         <v>18</v>
       </c>
@@ -2345,7 +2347,7 @@
         <v>3.6219561600085722E-2</v>
       </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
       <c r="E52" s="34" t="s">
         <v>19</v>
       </c>
@@ -2365,7 +2367,7 @@
         <v>3.7390996111162984E-2</v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="s">
         <v>49</v>
       </c>
@@ -2373,7 +2375,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B57" s="24" t="s">
         <v>35</v>
       </c>
@@ -2402,7 +2404,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B58" s="29" t="s">
         <v>36</v>
       </c>
@@ -2417,7 +2419,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G58" s="26" t="str" cm="1">
-        <f t="array" ref="G58">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F58,E58,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G58">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F58,E58,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R58C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I58" s="27" cm="1">
@@ -2425,7 +2427,7 @@
         <v>46541</v>
       </c>
       <c r="J58" s="28" cm="1">
-        <f t="array" ref="J58">_xll.qlYieldTermStructureZeroRate($C$73,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J58">_xll.qlYieldTermStructureZeroRate($C$74,I58,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>1.9056934878278965E-2</v>
       </c>
       <c r="L58" s="28" cm="1">
@@ -2433,11 +2435,11 @@
         <v>1.9423329540682495E-2</v>
       </c>
       <c r="M58" s="49">
-        <f>J58-L58</f>
+        <f t="shared" ref="M58:M65" si="0">J58-L58</f>
         <v>-3.6639466240353039E-4</v>
       </c>
     </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B59" s="29" t="s">
         <v>37</v>
       </c>
@@ -2451,7 +2453,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G59" s="31" t="str" cm="1">
-        <f t="array" ref="G59">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F59,E59,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G59">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F59,E59,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R59C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I59" s="32" cm="1">
@@ -2459,7 +2461,7 @@
         <v>46909</v>
       </c>
       <c r="J59" s="33" cm="1">
-        <f t="array" ref="J59">_xll.qlYieldTermStructureZeroRate($C$73,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J59">_xll.qlYieldTermStructureZeroRate($C$74,I59,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>1.9341237502176117E-2</v>
       </c>
       <c r="L59" s="33" cm="1">
@@ -2467,11 +2469,11 @@
         <v>1.9707419970420838E-2</v>
       </c>
       <c r="M59" s="50">
-        <f>J59-L59</f>
+        <f t="shared" si="0"/>
         <v>-3.6618246824472039E-4</v>
       </c>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B60" s="29" t="s">
         <v>47</v>
       </c>
@@ -2485,7 +2487,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G60" s="31" t="str" cm="1">
-        <f t="array" ref="G60">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F60,E60,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G60">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F60,E60,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R60C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I60" s="32" cm="1">
@@ -2493,7 +2495,7 @@
         <v>47273</v>
       </c>
       <c r="J60" s="33" cm="1">
-        <f t="array" ref="J60">_xll.qlYieldTermStructureZeroRate($C$73,I60,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J60">_xll.qlYieldTermStructureZeroRate($C$74,I60,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>1.9938542000702334E-2</v>
       </c>
       <c r="L60" s="33" cm="1">
@@ -2501,11 +2503,11 @@
         <v>2.0304501541429942E-2</v>
       </c>
       <c r="M60" s="50">
-        <f>J60-L60</f>
+        <f t="shared" si="0"/>
         <v>-3.6595954072760756E-4</v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B61" s="29" t="s">
         <v>39</v>
       </c>
@@ -2520,7 +2522,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G61" s="31" t="str" cm="1">
-        <f t="array" ref="G61">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F61,E61,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G61">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F61,E61,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R61C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I61" s="32" cm="1">
@@ -2528,7 +2530,7 @@
         <v>47637</v>
       </c>
       <c r="J61" s="33" cm="1">
-        <f t="array" ref="J61">_xll.qlYieldTermStructureZeroRate($C$73,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J61">_xll.qlYieldTermStructureZeroRate($C$74,I61,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>2.0690783526765087E-2</v>
       </c>
       <c r="L61" s="33" cm="1">
@@ -2536,11 +2538,11 @@
         <v>2.1056614418825545E-2</v>
       </c>
       <c r="M61" s="50">
-        <f>J61-L61</f>
+        <f t="shared" si="0"/>
         <v>-3.6583089206045777E-4</v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B62" s="29" t="s">
         <v>40</v>
       </c>
@@ -2555,7 +2557,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G62" s="31" t="str" cm="1">
-        <f t="array" ref="G62">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F62,E62,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G62">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F62,E62,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R62C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I62" s="32" cm="1">
@@ -2563,7 +2565,7 @@
         <v>48002</v>
       </c>
       <c r="J62" s="33" cm="1">
-        <f t="array" ref="J62">_xll.qlYieldTermStructureZeroRate($C$73,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J62">_xll.qlYieldTermStructureZeroRate($C$74,I62,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>2.1438592526394247E-2</v>
       </c>
       <c r="L62" s="33" cm="1">
@@ -2571,11 +2573,11 @@
         <v>2.1804311905509664E-2</v>
       </c>
       <c r="M62" s="50">
-        <f>J62-L62</f>
+        <f t="shared" si="0"/>
         <v>-3.657193791154166E-4</v>
       </c>
     </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B63" s="29" t="s">
         <v>41</v>
       </c>
@@ -2590,7 +2592,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G63" s="31" t="str" cm="1">
-        <f t="array" ref="G63">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F63,E63,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G63">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F63,E63,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R63C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I63" s="32" cm="1">
@@ -2598,7 +2600,7 @@
         <v>48733</v>
       </c>
       <c r="J63" s="33" cm="1">
-        <f t="array" ref="J63">_xll.qlYieldTermStructureZeroRate($C$73,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J63">_xll.qlYieldTermStructureZeroRate($C$74,I63,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>2.2939847920213422E-2</v>
       </c>
       <c r="L63" s="33" cm="1">
@@ -2606,11 +2608,11 @@
         <v>2.3305383398994673E-2</v>
       </c>
       <c r="M63" s="50">
-        <f>J63-L63</f>
+        <f t="shared" si="0"/>
         <v>-3.6553547878125092E-4</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B64" s="29" t="s">
         <v>42</v>
       </c>
@@ -2624,7 +2626,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G64" s="31" t="str" cm="1">
-        <f t="array" ref="G64">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F64,E64,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G64">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F64,E64,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R64C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I64" s="32" cm="1">
@@ -2632,7 +2634,7 @@
         <v>49829</v>
       </c>
       <c r="J64" s="33" cm="1">
-        <f t="array" ref="J64">_xll.qlYieldTermStructureZeroRate($C$73,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J64">_xll.qlYieldTermStructureZeroRate($C$74,I64,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>2.5029132269805833E-2</v>
       </c>
       <c r="L64" s="33" cm="1">
@@ -2640,11 +2642,11 @@
         <v>2.5394439430906784E-2</v>
       </c>
       <c r="M64" s="50">
-        <f>J64-L64</f>
+        <f t="shared" si="0"/>
         <v>-3.6530716110095077E-4</v>
       </c>
     </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B65" s="29" t="s">
         <v>43</v>
       </c>
@@ -2658,7 +2660,7 @@
         <v>-3.6249999999999998E-4</v>
       </c>
       <c r="G65" s="36" t="str" cm="1">
-        <f t="array" ref="G65">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F65,E65,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$3)</f>
+        <f t="array" ref="G65">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(F65,E65,$C$57,$C$58,$C$59,$C$60,$C$61,$C$62,$C$63,$C$64,$C$65,$C$66,$C$67,$C$68,$C$69,$C$3)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R65C7MtMCrossCurrencyBasisSwapRateHelper,A</v>
       </c>
       <c r="I65" s="37" cm="1">
@@ -2666,7 +2668,7 @@
         <v>50559</v>
       </c>
       <c r="J65" s="38" cm="1">
-        <f t="array" ref="J65">_xll.qlYieldTermStructureZeroRate($C$73,I65,"Act/365","Continuous","NoFrequency",TRUE)</f>
+        <f t="array" ref="J65">_xll.qlYieldTermStructureZeroRate($C$74,I65,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>2.6253758750164394E-2</v>
       </c>
       <c r="L65" s="38" cm="1">
@@ -2674,11 +2676,11 @@
         <v>2.6618940661949898E-2</v>
       </c>
       <c r="M65" s="51">
-        <f>J65-L65</f>
+        <f t="shared" si="0"/>
         <v>-3.6518191178550388E-4</v>
       </c>
     </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B66" s="29" t="s">
         <v>44</v>
       </c>
@@ -2686,7 +2688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B67" s="29" t="s">
         <v>45</v>
       </c>
@@ -2694,219 +2696,227 @@
         <v>46</v>
       </c>
     </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B68" s="34" t="s">
+    <row r="68" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B68" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="C68" s="54">
+      <c r="C68" s="42">
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B70" s="24" t="s">
+    <row r="69" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B69" s="34" t="s">
+        <v>173</v>
+      </c>
+      <c r="C69" s="43" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B71" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C70" s="41" t="s">
+      <c r="C71" s="41" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B71" s="29" t="s">
+    <row r="72" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B72" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C71" s="42" t="s">
+      <c r="C72" s="42" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B72" s="34" t="s">
+    <row r="73" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B73" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="C72" s="43" t="s">
+      <c r="C73" s="43" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B73" s="44" t="s">
+    <row r="74" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B74" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="C73" s="45" t="str" cm="1">
-        <f t="array" ref="C73">_xll.qlPiecewiseYieldCurve($C$3,G58:G65,C70,C71,C72)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Curves!R73C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B76" s="5" t="s">
+      <c r="C74" s="45" t="str" cm="1">
+        <f t="array" ref="C74">_xll.qlPiecewiseYieldCurve($C$3,G58:G65,C71,C72,C73)</f>
+        <v>欣[example_interest_rate_derivatives.xlsx]Curves!R74C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B77" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E76" s="5" t="s">
+      <c r="E77" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="78" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B78" s="24" t="s">
+    <row r="79" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B79" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C78" s="41" t="s">
+      <c r="C79" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E78" s="22" t="s">
+      <c r="E79" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F78" s="22" t="s">
+      <c r="F79" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="G78" s="44" t="s">
+      <c r="G79" s="44" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B79" s="29" t="s">
+    <row r="80" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B80" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C79" s="42" t="s">
+      <c r="C80" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="E79" s="55">
+      <c r="E80" s="54">
         <f>C3</f>
         <v>46174</v>
       </c>
-      <c r="F79" s="56" cm="1">
-        <f t="array" ref="F79">_xll.qlYieldTermStructureZeroRate($C$44,E79,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F80" s="55" cm="1">
+        <f t="array" ref="F80">_xll.qlYieldTermStructureZeroRate($C$44,E80,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.7513715269406556E-2</v>
       </c>
-      <c r="G79" s="49">
-        <f>F79-M58</f>
+      <c r="G80" s="49">
+        <f>F80-M58</f>
         <v>3.7880109931810083E-2</v>
       </c>
     </row>
-    <row r="80" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B80" s="34" t="s">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B81" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="C80" s="43" t="s">
+      <c r="C81" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="E80" s="57">
-        <f>I58</f>
+      <c r="E81" s="56">
+        <f t="shared" ref="E81:E88" si="1">I58</f>
         <v>46541</v>
       </c>
-      <c r="F80" s="58" cm="1">
-        <f t="array" ref="F80">_xll.qlYieldTermStructureZeroRate($C$44,E80,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F81" s="57" cm="1">
+        <f t="array" ref="F81">_xll.qlYieldTermStructureZeroRate($C$44,E81,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.4626290911888569E-2</v>
       </c>
-      <c r="G80" s="50">
-        <f>F80-M58</f>
+      <c r="G81" s="50">
+        <f>F81-M58</f>
         <v>3.4992685574292096E-2</v>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B81" s="44" t="s">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B82" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="C81" s="45" t="str" cm="1">
-        <f t="array" ref="C81">_xll.qlInterpolatedYieldCurve(E79:E87,G79:G87,C78,"NullCalendar",C79,C80)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Curves!R81C3YieldTermStructureHandle,A</v>
-      </c>
-      <c r="E81" s="57">
-        <f>I59</f>
+      <c r="C82" s="45" t="str" cm="1">
+        <f t="array" ref="C82">_xll.qlInterpolatedYieldCurve(E80:E88,G80:G88,C79,"NullCalendar",C80,C81)</f>
+        <v>欣[example_interest_rate_derivatives.xlsx]Curves!R82C3YieldTermStructureHandle,A</v>
+      </c>
+      <c r="E82" s="56">
+        <f t="shared" si="1"/>
         <v>46909</v>
       </c>
-      <c r="F81" s="58" cm="1">
-        <f t="array" ref="F81">_xll.qlYieldTermStructureZeroRate($C$44,E81,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F82" s="57" cm="1">
+        <f t="array" ref="F82">_xll.qlYieldTermStructureZeroRate($C$44,E82,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.2751768392570955E-2</v>
       </c>
-      <c r="G81" s="50">
-        <f>F81-M59</f>
+      <c r="G82" s="50">
+        <f>F82-M59</f>
         <v>3.3117950860815676E-2</v>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E82" s="57">
-        <f>I60</f>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E83" s="56">
+        <f t="shared" si="1"/>
         <v>47273</v>
       </c>
-      <c r="F82" s="58" cm="1">
-        <f t="array" ref="F82">_xll.qlYieldTermStructureZeroRate($C$44,E82,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F83" s="57" cm="1">
+        <f t="array" ref="F83">_xll.qlYieldTermStructureZeroRate($C$44,E83,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.2377367024610644E-2</v>
       </c>
-      <c r="G82" s="50">
-        <f>F82-M60</f>
+      <c r="G83" s="50">
+        <f>F83-M60</f>
         <v>3.2743326565338252E-2</v>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E83" s="57">
-        <f>I61</f>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E84" s="56">
+        <f t="shared" si="1"/>
         <v>47637</v>
       </c>
-      <c r="F83" s="58" cm="1">
-        <f t="array" ref="F83">_xll.qlYieldTermStructureZeroRate($C$44,E83,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F84" s="57" cm="1">
+        <f t="array" ref="F84">_xll.qlYieldTermStructureZeroRate($C$44,E84,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.2661635352545959E-2</v>
       </c>
-      <c r="G83" s="50">
-        <f>F83-M61</f>
+      <c r="G84" s="50">
+        <f>F84-M61</f>
         <v>3.3027466244606417E-2</v>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E84" s="57">
-        <f>I62</f>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E85" s="56">
+        <f t="shared" si="1"/>
         <v>48002</v>
       </c>
-      <c r="F84" s="58" cm="1">
-        <f t="array" ref="F84">_xll.qlYieldTermStructureZeroRate($C$44,E84,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F85" s="57" cm="1">
+        <f t="array" ref="F85">_xll.qlYieldTermStructureZeroRate($C$44,E85,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.3148897734764607E-2</v>
       </c>
-      <c r="G84" s="50">
-        <f>F84-M62</f>
+      <c r="G85" s="50">
+        <f>F85-M62</f>
         <v>3.3514617113880027E-2</v>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E85" s="57">
-        <f>I63</f>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E86" s="56">
+        <f t="shared" si="1"/>
         <v>48733</v>
       </c>
-      <c r="F85" s="58" cm="1">
-        <f t="array" ref="F85">_xll.qlYieldTermStructureZeroRate($C$44,E85,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F86" s="57" cm="1">
+        <f t="array" ref="F86">_xll.qlYieldTermStructureZeroRate($C$44,E86,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.4367701312975452E-2</v>
       </c>
-      <c r="G85" s="50">
-        <f>F85-M63</f>
+      <c r="G86" s="50">
+        <f>F86-M63</f>
         <v>3.4733236791756703E-2</v>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E86" s="57">
-        <f>I64</f>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E87" s="56">
+        <f t="shared" si="1"/>
         <v>49829</v>
       </c>
-      <c r="F86" s="58" cm="1">
-        <f t="array" ref="F86">_xll.qlYieldTermStructureZeroRate($C$44,E86,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F87" s="57" cm="1">
+        <f t="array" ref="F87">_xll.qlYieldTermStructureZeroRate($C$44,E87,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.6219561600085722E-2</v>
       </c>
-      <c r="G86" s="50">
-        <f>F86-M64</f>
+      <c r="G87" s="50">
+        <f>F87-M64</f>
         <v>3.6584868761186676E-2</v>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E87" s="59">
-        <f>I65</f>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E88" s="58">
+        <f t="shared" si="1"/>
         <v>50559</v>
       </c>
-      <c r="F87" s="60" cm="1">
-        <f t="array" ref="F87">_xll.qlYieldTermStructureZeroRate($C$44,E87,"Act/365","Continuous","NoFrequency",TRUE)</f>
+      <c r="F88" s="59" cm="1">
+        <f t="array" ref="F88">_xll.qlYieldTermStructureZeroRate($C$44,E88,"Act/365","Continuous","NoFrequency",TRUE)</f>
         <v>3.7390996111162984E-2</v>
       </c>
-      <c r="G87" s="51">
-        <f>F87-M65</f>
+      <c r="G88" s="51">
+        <f>F88-M65</f>
         <v>3.7756178022948492E-2</v>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E88" s="11"/>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E89" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2916,29 +2926,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA23A266-F08C-4F68-A68D-98AC63B9D7CD}">
   <dimension ref="B2:P64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="61">
+      <c r="C2" s="60">
         <f>Curves!C3</f>
         <v>46174</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>91</v>
       </c>
@@ -2946,7 +2956,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
         <v>59</v>
       </c>
@@ -2984,7 +2994,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>60</v>
       </c>
@@ -3024,11 +3034,11 @@
         <v>300.00000000000028</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="62" t="str" cm="1">
+      <c r="C8" s="61" t="str" cm="1">
         <f t="array" ref="C8">_xll.qlMakeSchedule(C6,C7,"1y",,"Target","Following")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R8C3Schedule,A</v>
       </c>
@@ -3063,7 +3073,7 @@
         <v>300.00000000000028</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="34" t="s">
         <v>65</v>
       </c>
@@ -3102,7 +3112,7 @@
         <v>301.66666666666674</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G10" s="2">
         <v>47609</v>
       </c>
@@ -3134,7 +3144,7 @@
         <v>299.16666666666589</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" s="24" t="s">
         <v>31</v>
       </c>
@@ -3173,11 +3183,11 @@
         <v>299.16666666666589</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="63" t="b" cm="1">
+      <c r="C12" s="62" t="b" cm="1">
         <f t="array" ref="C12">_xll.qlIndexAddFixing(C11,B13,C13,TRUE)</f>
         <v>1</v>
       </c>
@@ -3212,11 +3222,11 @@
         <v>300.00000000000028</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B13" s="64">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B13" s="63">
         <v>46142</v>
       </c>
-      <c r="C13" s="65">
+      <c r="C13" s="64">
         <v>2.1350000000000001E-2</v>
       </c>
       <c r="G13" s="2">
@@ -3250,7 +3260,7 @@
         <v>300.00000000000028</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G14" s="2">
         <v>49069</v>
       </c>
@@ -3282,7 +3292,7 @@
         <v>300.00000000000028</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B15" s="24" t="s">
         <v>76</v>
       </c>
@@ -3321,7 +3331,7 @@
         <v>301.66666666666674</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B16" s="34" t="s">
         <v>77</v>
       </c>
@@ -3360,10 +3370,10 @@
         <v>298.33333333333377</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="44" t="s">
         <v>78</v>
       </c>
@@ -3375,14 +3385,14 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="66" t="str">
+      <c r="C20" s="65" t="str">
         <f>Curves!C14</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R14C3YieldTermStructureHandle,A</v>
       </c>
@@ -3417,7 +3427,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="34" t="s">
         <v>79</v>
       </c>
@@ -3457,7 +3467,7 @@
         <v>109.12222222222222</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G22" s="2">
         <v>46512</v>
       </c>
@@ -3489,11 +3499,11 @@
         <v>107.51738481334705</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="67" cm="1">
+      <c r="C23" s="66" cm="1">
         <f t="array" ref="C23">_xll.qlInstrumentNPV(C18,_xll.qlInstrumentSetPricingEngine(C18,C21))</f>
         <v>-457.45759571020835</v>
       </c>
@@ -3528,7 +3538,7 @@
         <v>111.44985649460537</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G24" s="2">
         <v>46878</v>
       </c>
@@ -3560,7 +3570,7 @@
         <v>113.23641739098721</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G25" s="2">
         <v>47063</v>
       </c>
@@ -3592,7 +3602,7 @@
         <v>118.55587761160136</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>82</v>
       </c>
@@ -3627,7 +3637,7 @@
         <v>120.72760819356488</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G27" s="2">
         <v>47427</v>
       </c>
@@ -3659,11 +3669,11 @@
         <v>125.41837090147779</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B28" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="C28" s="70">
+      <c r="C28" s="69">
         <v>0</v>
       </c>
       <c r="G28" s="2">
@@ -3697,11 +3707,11 @@
         <v>129.21427943945352</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="C29" s="71">
+      <c r="C29" s="70">
         <v>0.03</v>
       </c>
       <c r="G29" s="2">
@@ -3735,11 +3745,11 @@
         <v>132.49026757669702</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="C30" s="69">
+      <c r="C30" s="68">
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="G30" s="2">
@@ -3773,7 +3783,7 @@
         <v>133.79883823478212</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>87</v>
       </c>
@@ -3812,7 +3822,7 @@
         <v>139.59904306338979</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>88</v>
       </c>
@@ -3851,7 +3861,7 @@
         <v>141.74364792127747</v>
       </c>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="34" t="s">
         <v>89</v>
       </c>
@@ -3890,7 +3900,7 @@
         <v>146.91955609455354</v>
       </c>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G34" s="2">
         <v>48704</v>
       </c>
@@ -3922,7 +3932,7 @@
         <v>147.94045035310123</v>
       </c>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B35" s="22" t="s">
         <v>85</v>
       </c>
@@ -3961,7 +3971,7 @@
         <v>155.48098106948683</v>
       </c>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G36" s="2">
         <v>49069</v>
       </c>
@@ -3993,8 +4003,8 @@
         <v>152.63586644126858</v>
       </c>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B37" s="72" t="str" cm="1">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B37" s="71" t="str" cm="1">
         <f t="array" ref="B37:B56">_xll.xloVal(C16)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,A</v>
       </c>
@@ -4033,8 +4043,8 @@
         <v>160.66149489961214</v>
       </c>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B38" s="73" t="str">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B38" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,B</v>
       </c>
       <c r="C38" s="31" t="str" cm="1">
@@ -4072,8 +4082,8 @@
         <v>160.6089850120207</v>
       </c>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B39" s="73" t="str">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B39" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,C</v>
       </c>
       <c r="C39" s="31" t="str" cm="1">
@@ -4111,8 +4121,8 @@
         <v>162.8898701505621</v>
       </c>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="73" t="str">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B40" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,D</v>
       </c>
       <c r="C40" s="31" t="str" cm="1">
@@ -4150,8 +4160,8 @@
         <v>164.90068665729441</v>
       </c>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B41" s="73" t="str">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B41" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,E</v>
       </c>
       <c r="C41" s="31" t="str" cm="1">
@@ -4159,8 +4169,8 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R41C3CappedFlooredCoupon,A</v>
       </c>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B42" s="73" t="str">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B42" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,F</v>
       </c>
       <c r="C42" s="31" t="str" cm="1">
@@ -4171,8 +4181,8 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B43" s="73" t="str">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B43" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,G</v>
       </c>
       <c r="C43" s="31" t="str" cm="1">
@@ -4180,8 +4190,8 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R43C3CappedFlooredCoupon,A</v>
       </c>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B44" s="73" t="str">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B44" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,H</v>
       </c>
       <c r="C44" s="31" t="str" cm="1">
@@ -4219,8 +4229,8 @@
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B45" s="73" t="str">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B45" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,I</v>
       </c>
       <c r="C45" s="31" t="str" cm="1">
@@ -4259,8 +4269,8 @@
         <v>109.12222222222222</v>
       </c>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B46" s="73" t="str">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B46" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,J</v>
       </c>
       <c r="C46" s="31" t="str" cm="1">
@@ -4298,8 +4308,8 @@
         <v>106.9799204944642</v>
       </c>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B47" s="73" t="str">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B47" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,K</v>
       </c>
       <c r="C47" s="31" t="str" cm="1">
@@ -4337,8 +4347,8 @@
         <v>108.60695689450282</v>
       </c>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B48" s="73" t="str">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B48" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,L</v>
       </c>
       <c r="C48" s="31" t="str" cm="1">
@@ -4376,8 +4386,8 @@
         <v>107.54785024681529</v>
       </c>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B49" s="73" t="str">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B49" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,M</v>
       </c>
       <c r="C49" s="31" t="str" cm="1">
@@ -4415,8 +4425,8 @@
         <v>109.70835521544075</v>
       </c>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B50" s="73" t="str">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B50" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,N</v>
       </c>
       <c r="C50" s="31" t="str" cm="1">
@@ -4454,8 +4464,8 @@
         <v>108.76651438463294</v>
       </c>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B51" s="73" t="str">
+    <row r="51" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B51" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,O</v>
       </c>
       <c r="C51" s="31" t="str" cm="1">
@@ -4493,8 +4503,8 @@
         <v>109.94523667689172</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B52" s="73" t="str">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B52" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,P</v>
       </c>
       <c r="C52" s="31" t="str" cm="1">
@@ -4532,8 +4542,8 @@
         <v>110.53963553262899</v>
       </c>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B53" s="73" t="str">
+    <row r="53" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B53" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,Q</v>
       </c>
       <c r="C53" s="31" t="str" cm="1">
@@ -4571,8 +4581,8 @@
         <v>111.06503376964604</v>
       </c>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="73" t="str">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B54" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,R</v>
       </c>
       <c r="C54" s="31" t="str" cm="1">
@@ -4610,8 +4620,8 @@
         <v>109.94246375047065</v>
       </c>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="73" t="str">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B55" s="72" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,S</v>
       </c>
       <c r="C55" s="31" t="str" cm="1">
@@ -4649,8 +4659,8 @@
         <v>112.31140449604059</v>
       </c>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B56" s="74" t="str">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B56" s="73" t="str">
         <v>欣[example_interest_rate_derivatives.xlsx]Euribor swap!R16C3CashFlow,T</v>
       </c>
       <c r="C56" s="36" t="str" cm="1">
@@ -4688,7 +4698,7 @@
         <v>111.64164254928934</v>
       </c>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G57" s="2">
         <v>48523</v>
       </c>
@@ -4720,7 +4730,7 @@
         <v>113.41461849761878</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G58" s="2">
         <v>48704</v>
       </c>
@@ -4752,7 +4762,7 @@
         <v>112.02384372239797</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G59" s="2">
         <v>48890</v>
       </c>
@@ -4784,7 +4794,7 @@
         <v>115.58167475666409</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G60" s="2">
         <v>49069</v>
       </c>
@@ -4816,7 +4826,7 @@
         <v>111.53154008736583</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G61" s="2">
         <v>49254</v>
       </c>
@@ -4848,7 +4858,7 @@
         <v>115.52378989666693</v>
       </c>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G62" s="2">
         <v>49436</v>
       </c>
@@ -4880,7 +4890,7 @@
         <v>113.78062080563485</v>
       </c>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G63" s="2">
         <v>49618</v>
       </c>
@@ -4912,7 +4922,7 @@
         <v>113.82751042427807</v>
       </c>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G64" s="2">
         <v>49800</v>
       </c>
@@ -4952,29 +4962,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{877F551F-FE76-4C1A-99E8-54C3F83BB0FF}">
   <dimension ref="B2:P55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="61">
+      <c r="C2" s="60">
         <f>Curves!C3</f>
         <v>46174</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>91</v>
       </c>
@@ -4982,7 +4992,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
         <v>59</v>
       </c>
@@ -5020,7 +5030,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>60</v>
       </c>
@@ -5060,11 +5070,11 @@
         <v>94.137296800429482</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="75" t="str" cm="1">
+      <c r="C8" s="74" t="str" cm="1">
         <f t="array" ref="C8">_xll.qlMakeSchedule(C6,C7,"3m",,"NYC","Following")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Sofr swap!R8C3Schedule,A</v>
       </c>
@@ -5099,7 +5109,7 @@
         <v>91.59212079587364</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C9" s="4"/>
       <c r="G9" s="2">
         <v>46422</v>
@@ -5132,7 +5142,7 @@
         <v>86.752204299058718</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" s="23" t="s">
         <v>170</v>
       </c>
@@ -5171,7 +5181,7 @@
         <v>79.523130991412387</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G11" s="2">
         <v>46603</v>
       </c>
@@ -5203,7 +5213,7 @@
         <v>79.709499892377522</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" s="24" t="s">
         <v>92</v>
       </c>
@@ -5242,7 +5252,7 @@
         <v>78.354180805149113</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>93</v>
       </c>
@@ -5281,7 +5291,7 @@
         <v>79.349828668098255</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B14" s="34" t="s">
         <v>94</v>
       </c>
@@ -5320,7 +5330,7 @@
         <v>74.223001504190037</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G15" s="2">
         <v>46969</v>
       </c>
@@ -5352,7 +5362,7 @@
         <v>79.888424280218914</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C16" s="3"/>
       <c r="G16" s="2">
         <v>47060</v>
@@ -5385,7 +5395,7 @@
         <v>78.231611636114806</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="7" t="s">
         <v>95</v>
       </c>
@@ -5421,7 +5431,7 @@
         <v>79.268803223127009</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C18" s="3"/>
       <c r="G18" s="2">
         <v>47242</v>
@@ -5454,7 +5464,7 @@
         <v>80.450585469296072</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="24" t="s">
         <v>171</v>
       </c>
@@ -5493,7 +5503,7 @@
         <v>81.762246846175387</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="34" t="s">
         <v>64</v>
       </c>
@@ -5532,7 +5542,7 @@
         <v>83.047242778340191</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G21" s="2">
         <v>47518</v>
       </c>
@@ -5564,11 +5574,11 @@
         <v>85.146572110013082</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="76" t="s">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B22" s="75" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="76" t="s">
+      <c r="C22" s="75" t="s">
         <v>63</v>
       </c>
       <c r="G22" s="2">
@@ -5602,12 +5612,12 @@
         <v>84.317537287457171</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="27" cm="1">
         <f t="array" ref="B23:B41">_xll.qlScheduleDates(C19,C12)</f>
         <v>46147</v>
       </c>
-      <c r="C23" s="77">
+      <c r="C23" s="76">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G23" s="2">
@@ -5641,11 +5651,11 @@
         <v>86.181408898644563</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="32">
         <v>46148</v>
       </c>
-      <c r="C24" s="78">
+      <c r="C24" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G24" s="2">
@@ -5679,11 +5689,11 @@
         <v>88.061473562544009</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B25" s="32">
         <v>46149</v>
       </c>
-      <c r="C25" s="78">
+      <c r="C25" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G25" s="2">
@@ -5717,11 +5727,11 @@
         <v>89.040916820186666</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="32">
         <v>46150</v>
       </c>
-      <c r="C26" s="78">
+      <c r="C26" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G26" s="2">
@@ -5755,11 +5765,11 @@
         <v>87.100458544671085</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B27" s="32">
         <v>46153</v>
       </c>
-      <c r="C27" s="78">
+      <c r="C27" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G27" s="2">
@@ -5793,11 +5803,11 @@
         <v>91.098711779020732</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B28" s="32">
         <v>46154</v>
       </c>
-      <c r="C28" s="78">
+      <c r="C28" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G28" s="2">
@@ -5831,11 +5841,11 @@
         <v>92.153932954790463</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B29" s="32">
         <v>46155</v>
       </c>
-      <c r="C29" s="78">
+      <c r="C29" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G29" s="2">
@@ -5869,11 +5879,11 @@
         <v>93.166021778989801</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B30" s="32">
         <v>46156</v>
       </c>
-      <c r="C30" s="78">
+      <c r="C30" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G30" s="2">
@@ -5907,11 +5917,11 @@
         <v>92.068710436405965</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B31" s="32">
         <v>46157</v>
       </c>
-      <c r="C31" s="78">
+      <c r="C31" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G31" s="2">
@@ -5945,11 +5955,11 @@
         <v>95.039698270384946</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B32" s="32">
         <v>46160</v>
       </c>
-      <c r="C32" s="78">
+      <c r="C32" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G32" s="2">
@@ -5983,11 +5993,11 @@
         <v>95.921851504920937</v>
       </c>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="32">
         <v>46161</v>
       </c>
-      <c r="C33" s="78">
+      <c r="C33" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G33" s="2">
@@ -6021,11 +6031,11 @@
         <v>98.883191699234985</v>
       </c>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B34" s="32">
         <v>46162</v>
       </c>
-      <c r="C34" s="78">
+      <c r="C34" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G34" s="2">
@@ -6059,11 +6069,11 @@
         <v>92.225118139901411</v>
       </c>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B35" s="32">
         <v>46163</v>
       </c>
-      <c r="C35" s="78">
+      <c r="C35" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G35" s="2">
@@ -6097,11 +6107,11 @@
         <v>98.285267460855863</v>
       </c>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B36" s="32">
         <v>46164</v>
       </c>
-      <c r="C36" s="78">
+      <c r="C36" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G36" s="2">
@@ -6135,11 +6145,11 @@
         <v>101.20114794352597</v>
       </c>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B37" s="32">
         <v>46168</v>
       </c>
-      <c r="C37" s="78">
+      <c r="C37" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G37" s="2">
@@ -6173,11 +6183,11 @@
         <v>98.702100763499175</v>
       </c>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B38" s="32">
         <v>46169</v>
       </c>
-      <c r="C38" s="78">
+      <c r="C38" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G38" s="2">
@@ -6211,11 +6221,11 @@
         <v>96.137471482982136</v>
       </c>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B39" s="32">
         <v>46170</v>
       </c>
-      <c r="C39" s="78">
+      <c r="C39" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G39" s="2">
@@ -6249,11 +6259,11 @@
         <v>103.49882101314822</v>
       </c>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B40" s="32">
         <v>46171</v>
       </c>
-      <c r="C40" s="78">
+      <c r="C40" s="77">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G40" s="2">
@@ -6287,11 +6297,11 @@
         <v>100.94648181865563</v>
       </c>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B41" s="37">
         <v>46174</v>
       </c>
-      <c r="C41" s="79">
+      <c r="C41" s="78">
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="G41" s="2">
@@ -6325,7 +6335,7 @@
         <v>101.70822893849297</v>
       </c>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C42" s="3"/>
       <c r="G42" s="2">
         <v>49433</v>
@@ -6358,7 +6368,7 @@
         <v>102.47678865155319</v>
       </c>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C43" s="3"/>
       <c r="G43" s="2">
         <v>49524</v>
@@ -6391,7 +6401,7 @@
         <v>103.25216250400837</v>
       </c>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C44" s="3"/>
       <c r="G44" s="2">
         <v>49615</v>
@@ -6424,7 +6434,7 @@
         <v>104.03435205581957</v>
       </c>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C45" s="3"/>
       <c r="G45" s="2">
         <v>49709</v>
@@ -6457,7 +6467,7 @@
         <v>105.98575529064293</v>
       </c>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C46" s="3"/>
       <c r="G46" s="2">
         <v>49797</v>
@@ -6490,31 +6500,31 @@
         <v>104.45683031957253</v>
       </c>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C47" s="3"/>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C48" s="3"/>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C49" s="3"/>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C50" s="3"/>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C51" s="3"/>
     </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C52" s="3"/>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C53" s="3"/>
     </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C54" s="3"/>
     </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C55" s="3"/>
     </row>
   </sheetData>
@@ -6525,81 +6535,81 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9C7E61A-F9E2-4AFA-9E46-1C6AC5ED8AF2}">
   <dimension ref="B2:X64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.44140625" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.28515625" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.7109375" customWidth="1"/>
-    <col min="24" max="24" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.33203125" customWidth="1"/>
+    <col min="20" max="20" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.6640625" customWidth="1"/>
+    <col min="24" max="24" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="61">
+      <c r="C2" s="60">
         <f>Curves!C3</f>
         <v>46174</v>
       </c>
       <c r="E2" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="94" t="s">
+      <c r="F2" s="93" t="s">
         <v>97</v>
       </c>
-      <c r="G2" s="95" t="s">
+      <c r="G2" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="H2" s="95" t="s">
+      <c r="H2" s="94" t="s">
         <v>99</v>
       </c>
-      <c r="I2" s="95" t="s">
+      <c r="I2" s="94" t="s">
         <v>100</v>
       </c>
-      <c r="J2" s="95" t="s">
+      <c r="J2" s="94" t="s">
         <v>101</v>
       </c>
-      <c r="K2" s="96" t="s">
+      <c r="K2" s="95" t="s">
         <v>102</v>
       </c>
       <c r="L2" s="22" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E3" s="97" t="s">
+    <row r="3" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E3" s="96" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="100">
+      <c r="F3" s="99">
         <v>7.3156703444470991E-3</v>
       </c>
-      <c r="G3" s="101">
+      <c r="G3" s="100">
         <v>7.3545191823137079E-3</v>
       </c>
-      <c r="H3" s="101">
+      <c r="H3" s="100">
         <v>7.2034359041569691E-3</v>
       </c>
-      <c r="I3" s="101">
+      <c r="I3" s="100">
         <v>7.0085770171602179E-3</v>
       </c>
-      <c r="J3" s="101">
+      <c r="J3" s="100">
         <v>6.8685932674608981E-3</v>
       </c>
-      <c r="K3" s="102">
+      <c r="K3" s="101">
         <v>6.7945145206867591E-3</v>
       </c>
       <c r="L3" s="27" cm="1">
@@ -6607,33 +6617,33 @@
         <v>46905</v>
       </c>
     </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B4" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="C4" s="80" t="str">
+      <c r="C4" s="79" t="str">
         <f>Curves!C44</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R44C3YieldTermStructureHandle,A</v>
       </c>
-      <c r="E4" s="98" t="s">
+      <c r="E4" s="97" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="103">
+      <c r="F4" s="102">
         <v>7.3156703444470991E-3</v>
       </c>
-      <c r="G4" s="104">
+      <c r="G4" s="103">
         <v>7.3545191823137079E-3</v>
       </c>
-      <c r="H4" s="104">
+      <c r="H4" s="103">
         <v>7.2034359041569691E-3</v>
       </c>
-      <c r="I4" s="104">
+      <c r="I4" s="103">
         <v>7.0085770171602179E-3</v>
       </c>
-      <c r="J4" s="104">
+      <c r="J4" s="103">
         <v>6.8685932674608981E-3</v>
       </c>
-      <c r="K4" s="105">
+      <c r="K4" s="104">
         <v>6.7609933594352887E-3</v>
       </c>
       <c r="L4" s="32" cm="1">
@@ -6641,7 +6651,7 @@
         <v>47270</v>
       </c>
     </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B5" s="29" t="s">
         <v>108</v>
       </c>
@@ -6649,25 +6659,25 @@
         <f t="array" ref="C5">_xll.qlSwaptionVolatilityMatrix(C2,L3:L11,F2:K2,F3:K11,"Act/365",TRUE,"Normal",,C2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R5C3SwaptionVolatilityStructureHandle,A</v>
       </c>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="97" t="s">
         <v>104</v>
       </c>
-      <c r="F5" s="103">
+      <c r="F5" s="102">
         <v>7.2817581863660278E-3</v>
       </c>
-      <c r="G5" s="104">
+      <c r="G5" s="103">
         <v>7.2696284121221786E-3</v>
       </c>
-      <c r="H5" s="104">
+      <c r="H5" s="103">
         <v>7.1304987601498587E-3</v>
       </c>
-      <c r="I5" s="104">
+      <c r="I5" s="103">
         <v>6.9283035181297286E-3</v>
       </c>
-      <c r="J5" s="104">
+      <c r="J5" s="103">
         <v>6.8008276595723591E-3</v>
       </c>
-      <c r="K5" s="105">
+      <c r="K5" s="104">
         <v>6.667429100858718E-3</v>
       </c>
       <c r="L5" s="32" cm="1">
@@ -6675,7 +6685,7 @@
         <v>47637</v>
       </c>
     </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>122</v>
       </c>
@@ -6683,25 +6693,25 @@
         <f t="array" ref="C6">_xll.qlDiscountingSwapEngine(C4,FALSE)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R6C3DiscountingSwapEngine,A</v>
       </c>
-      <c r="E6" s="98" t="s">
+      <c r="E6" s="97" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="103">
+      <c r="F6" s="102">
         <v>7.2127847115574777E-3</v>
       </c>
-      <c r="G6" s="104">
+      <c r="G6" s="103">
         <v>7.2041310210440683E-3</v>
       </c>
-      <c r="H6" s="104">
+      <c r="H6" s="103">
         <v>7.0263612417479082E-3</v>
       </c>
-      <c r="I6" s="104">
+      <c r="I6" s="103">
         <v>6.8299999999999993E-3</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="103">
         <v>6.7098768442212988E-3</v>
       </c>
-      <c r="K6" s="105">
+      <c r="K6" s="104">
         <v>6.5734245883187388E-3</v>
       </c>
       <c r="L6" s="32" cm="1">
@@ -6709,7 +6719,7 @@
         <v>48001</v>
       </c>
     </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B7" s="34" t="s">
         <v>121</v>
       </c>
@@ -6717,25 +6727,25 @@
         <f t="array" ref="C7">_xll.qlBachelierSwaptionEngine(C4,C5)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R7C3BachelierSwaptionEngine,A</v>
       </c>
-      <c r="E7" s="98" t="s">
+      <c r="E7" s="97" t="s">
         <v>105</v>
       </c>
-      <c r="F7" s="103">
+      <c r="F7" s="102">
         <v>7.1067227208732493E-3</v>
       </c>
-      <c r="G7" s="104">
+      <c r="G7" s="103">
         <v>7.0954835416969491E-3</v>
       </c>
-      <c r="H7" s="104">
+      <c r="H7" s="103">
         <v>6.9032080676596688E-3</v>
       </c>
-      <c r="I7" s="104">
+      <c r="I7" s="103">
         <v>6.6952517114972181E-3</v>
       </c>
-      <c r="J7" s="104">
+      <c r="J7" s="103">
         <v>6.5607795355508477E-3</v>
       </c>
-      <c r="K7" s="105">
+      <c r="K7" s="104">
         <v>6.4205016338086587E-3</v>
       </c>
       <c r="L7" s="32" cm="1">
@@ -6743,26 +6753,26 @@
         <v>48366</v>
       </c>
     </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E8" s="98" t="s">
+    <row r="8" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E8" s="97" t="s">
         <v>101</v>
       </c>
-      <c r="F8" s="103">
+      <c r="F8" s="102">
         <v>6.9935462562427386E-3</v>
       </c>
-      <c r="G8" s="104">
+      <c r="G8" s="103">
         <v>6.9834102491734378E-3</v>
       </c>
-      <c r="H8" s="104">
+      <c r="H8" s="103">
         <v>6.7802047066821882E-3</v>
       </c>
-      <c r="I8" s="104">
+      <c r="I8" s="103">
         <v>6.5598608899994481E-3</v>
       </c>
-      <c r="J8" s="104">
+      <c r="J8" s="103">
         <v>6.408766326632169E-3</v>
       </c>
-      <c r="K8" s="105">
+      <c r="K8" s="104">
         <v>6.2645776071992877E-3</v>
       </c>
       <c r="L8" s="32" cm="1">
@@ -6770,26 +6780,26 @@
         <v>48731</v>
       </c>
     </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E9" s="98" t="s">
+    <row r="9" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E9" s="97" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="103">
+      <c r="F9" s="102">
         <v>6.8407381849624888E-3</v>
       </c>
-      <c r="G9" s="104">
+      <c r="G9" s="103">
         <v>6.8608351762795578E-3</v>
       </c>
-      <c r="H9" s="104">
+      <c r="H9" s="103">
         <v>6.6571986033943584E-3</v>
       </c>
-      <c r="I9" s="104">
+      <c r="I9" s="103">
         <v>6.4157223331967883E-3</v>
       </c>
-      <c r="J9" s="104">
+      <c r="J9" s="103">
         <v>6.2640620876668589E-3</v>
       </c>
-      <c r="K9" s="105">
+      <c r="K9" s="104">
         <v>6.0960353967729093E-3</v>
       </c>
       <c r="L9" s="32" cm="1">
@@ -6797,26 +6807,26 @@
         <v>49096</v>
       </c>
     </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E10" s="98" t="s">
+    <row r="10" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E10" s="97" t="s">
         <v>107</v>
       </c>
-      <c r="F10" s="103">
+      <c r="F10" s="102">
         <v>6.785482664909798E-3</v>
       </c>
-      <c r="G10" s="104">
+      <c r="G10" s="103">
         <v>6.7661093849715487E-3</v>
       </c>
-      <c r="H10" s="104">
+      <c r="H10" s="103">
         <v>6.554176344910399E-3</v>
       </c>
-      <c r="I10" s="104">
+      <c r="I10" s="103">
         <v>6.2951067334708986E-3</v>
       </c>
-      <c r="J10" s="104">
+      <c r="J10" s="103">
         <v>6.1192589232749693E-3</v>
       </c>
-      <c r="K10" s="105">
+      <c r="K10" s="104">
         <v>5.9343809605290482E-3</v>
       </c>
       <c r="L10" s="32" cm="1">
@@ -6824,26 +6834,26 @@
         <v>49461</v>
       </c>
     </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E11" s="99" t="s">
+    <row r="11" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E11" s="98" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="106">
+      <c r="F11" s="105">
         <v>6.6471299594392692E-3</v>
       </c>
-      <c r="G11" s="107">
+      <c r="G11" s="106">
         <v>6.6550559406967393E-3</v>
       </c>
-      <c r="H11" s="107">
+      <c r="H11" s="106">
         <v>6.4498956923306483E-3</v>
       </c>
-      <c r="I11" s="107">
+      <c r="I11" s="106">
         <v>6.1746353255577487E-3</v>
       </c>
-      <c r="J11" s="107">
+      <c r="J11" s="106">
         <v>5.9884341705214589E-3</v>
       </c>
-      <c r="K11" s="108">
+      <c r="K11" s="107">
         <v>5.7827242854212382E-3</v>
       </c>
       <c r="L11" s="37" cm="1">
@@ -6851,86 +6861,86 @@
         <v>49828</v>
       </c>
     </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B14" s="123" t="s">
+    <row r="14" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="B14" s="122" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="54">
         <f>'Sofr swap'!C6</f>
         <v>46147</v>
       </c>
-      <c r="E16" s="76" t="s">
+      <c r="E16" s="75" t="s">
         <v>111</v>
       </c>
-      <c r="F16" s="76" t="s">
+      <c r="F16" s="75" t="s">
         <v>110</v>
       </c>
-      <c r="G16" s="76" t="s">
+      <c r="G16" s="75" t="s">
         <v>114</v>
       </c>
-      <c r="H16" s="76" t="s">
+      <c r="H16" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="I16" s="76" t="s">
+      <c r="I16" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="J16" s="76" t="s">
+      <c r="J16" s="75" t="s">
         <v>123</v>
       </c>
-      <c r="K16" s="76" t="s">
+      <c r="K16" s="75" t="s">
         <v>109</v>
       </c>
-      <c r="L16" s="76" t="s">
+      <c r="L16" s="75" t="s">
         <v>112</v>
       </c>
-      <c r="M16" s="76" t="s">
+      <c r="M16" s="75" t="s">
         <v>113</v>
       </c>
-      <c r="N16" s="76" t="s">
+      <c r="N16" s="75" t="s">
         <v>123</v>
       </c>
-      <c r="O16" s="76" t="s">
+      <c r="O16" s="75" t="s">
         <v>124</v>
       </c>
-      <c r="Q16" s="76" t="s">
+      <c r="Q16" s="75" t="s">
         <v>86</v>
       </c>
-      <c r="R16" s="76" t="s">
+      <c r="R16" s="75" t="s">
         <v>151</v>
       </c>
-      <c r="S16" s="76" t="s">
+      <c r="S16" s="75" t="s">
         <v>125</v>
       </c>
-      <c r="T16" s="76" t="s">
+      <c r="T16" s="75" t="s">
         <v>126</v>
       </c>
-      <c r="U16" s="76" t="s">
+      <c r="U16" s="75" t="s">
         <v>127</v>
       </c>
-      <c r="V16" s="76" t="s">
+      <c r="V16" s="75" t="s">
         <v>128</v>
       </c>
-      <c r="W16" s="76" t="s">
+      <c r="W16" s="75" t="s">
         <v>133</v>
       </c>
-      <c r="X16" s="76" t="s">
+      <c r="X16" s="75" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="57">
+      <c r="C17" s="56">
         <f>'Sofr swap'!C7</f>
         <v>49800</v>
       </c>
-      <c r="E17" s="87" t="s">
+      <c r="E17" s="86" t="s">
         <v>97</v>
       </c>
       <c r="F17" s="27" cm="1">
@@ -6947,9 +6957,9 @@
       </c>
       <c r="I17" s="26" t="str" cm="1">
         <f t="array" ref="I17">_xll.qlOvernightIndexedSwap("Payer",$C$21,H17,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C9OvernightIndexedSwap,G</v>
-      </c>
-      <c r="J17" s="109" cm="1">
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C9OvernightIndexedSwap,A</v>
+      </c>
+      <c r="J17" s="108" cm="1">
         <f t="array" ref="J17">_xll.qlSwapLegBPS(I17,1,_xll.qlInstrumentSetPricingEngine(I17,$C$6))*10000</f>
         <v>75803.2600393584</v>
       </c>
@@ -6961,11 +6971,11 @@
         <f t="array" ref="L17">_xll.qlSwaption(I17,K17,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C12Swaption,A</v>
       </c>
-      <c r="M17" s="88" cm="1">
+      <c r="M17" s="87" cm="1">
         <f t="array" ref="M17">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$7))</f>
         <v>480.19741230417134</v>
       </c>
-      <c r="N17" s="109" cm="1">
+      <c r="N17" s="108" cm="1">
         <f t="array" ref="N17">_xll.qlSwaptionAnnuity(L17,M17)</f>
         <v>75803.2600393584</v>
       </c>
@@ -6977,26 +6987,26 @@
         <f t="array" ref="Q17">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F17,S17,$C$22)</f>
         <v>6.8192074362781394E-3</v>
       </c>
-      <c r="R17" s="112">
-        <f>G17-F17</f>
+      <c r="R17" s="111">
+        <f t="shared" ref="R17:R25" si="0">G17-F17</f>
         <v>2</v>
       </c>
-      <c r="S17" s="113" t="str">
-        <f>ROUND(($C$17-G17)/365.25,0)&amp;"y"</f>
+      <c r="S17" s="112" t="str">
+        <f t="shared" ref="S17:S25" si="1">ROUND(($C$17-G17)/365.25,0)&amp;"y"</f>
         <v>9y</v>
       </c>
       <c r="T17" s="26" t="str" cm="1">
         <f t="array" ref="T17">_xll.qlSwaptionHelper(F17,S17,Q17,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R17,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C20SwaptionHelper,A</v>
       </c>
-      <c r="U17" s="68">
+      <c r="U17" s="67">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V17" s="114">
-        <f>$C$30</f>
+      <c r="V17" s="113">
+        <f t="shared" ref="V17:V26" si="2">$C$30</f>
         <v>0.01</v>
       </c>
-      <c r="W17" s="115" t="b" cm="1">
+      <c r="W17" s="114" t="b" cm="1">
         <f t="array" ref="W17">_xll.qlBlackCalibrationHelperSetPricingEngine(T17,$C$32)</f>
         <v>1</v>
       </c>
@@ -7005,7 +7015,7 @@
         <v>7.2562982901529325E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>115</v>
       </c>
@@ -7013,7 +7023,7 @@
         <f>'Sofr swap'!C14</f>
         <v>永[example_interest_rate_derivatives.xlsx]Sofr swap!R14C3,A</v>
       </c>
-      <c r="E18" s="98" t="s">
+      <c r="E18" s="97" t="s">
         <v>98</v>
       </c>
       <c r="F18" s="32" cm="1">
@@ -7032,7 +7042,7 @@
         <f t="array" ref="I18">_xll.qlOvernightIndexedSwap("Payer",$C$21,H18,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J18" s="110" cm="1">
+      <c r="J18" s="109" cm="1">
         <f t="array" ref="J18">_xll.qlSwapLegBPS(I18,1,_xll.qlInstrumentSetPricingEngine(I18,$C$6))*10000</f>
         <v>66149.320380348523</v>
       </c>
@@ -7044,11 +7054,11 @@
         <f t="array" ref="L18">_xll.qlSwaption(I18,K18,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C12Swaption,A</v>
       </c>
-      <c r="M18" s="90" cm="1">
+      <c r="M18" s="89" cm="1">
         <f t="array" ref="M18">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$7))</f>
         <v>514.76204370168534</v>
       </c>
-      <c r="N18" s="110" cm="1">
+      <c r="N18" s="109" cm="1">
         <f t="array" ref="N18">_xll.qlSwaptionAnnuity(L18,M18)</f>
         <v>66149.320380348523</v>
       </c>
@@ -7060,26 +7070,26 @@
         <f t="array" ref="Q18">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F18,S18,$C$22)</f>
         <v>6.8439003518695187E-3</v>
       </c>
-      <c r="R18" s="116">
-        <f>G18-F18</f>
+      <c r="R18" s="115">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="S18" s="117" t="str">
-        <f>ROUND(($C$17-G18)/365.25,0)&amp;"y"</f>
+      <c r="S18" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>8y</v>
       </c>
       <c r="T18" s="31" t="str" cm="1">
         <f t="array" ref="T18">_xll.qlSwaptionHelper(F18,S18,Q18,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R18,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C20SwaptionHelper,A</v>
       </c>
-      <c r="U18" s="69">
+      <c r="U18" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V18" s="118">
-        <f>$C$30</f>
+      <c r="V18" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W18" s="63" t="b" cm="1">
+      <c r="W18" s="62" t="b" cm="1">
         <f t="array" ref="W18">_xll.qlBlackCalibrationHelperSetPricingEngine(T18,$C$32)</f>
         <v>1</v>
       </c>
@@ -7087,15 +7097,15 @@
         <v>7.2854447762798731E-3</v>
       </c>
     </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B19" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="81" t="str">
+      <c r="C19" s="80" t="str">
         <f>'Sofr swap'!C10</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Sofr swap!R10C3Sofr,A</v>
       </c>
-      <c r="E19" s="98" t="s">
+      <c r="E19" s="97" t="s">
         <v>99</v>
       </c>
       <c r="F19" s="32" cm="1">
@@ -7114,7 +7124,7 @@
         <f t="array" ref="I19">_xll.qlOvernightIndexedSwap("Payer",$C$21,H19,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J19" s="110" cm="1">
+      <c r="J19" s="109" cm="1">
         <f t="array" ref="J19">_xll.qlSwapLegBPS(I19,1,_xll.qlInstrumentSetPricingEngine(I19,$C$6))*10000</f>
         <v>56766.422970738095</v>
       </c>
@@ -7126,11 +7136,11 @@
         <f t="array" ref="L19">_xll.qlSwaption(I19,K19,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C12Swaption,A</v>
       </c>
-      <c r="M19" s="90" cm="1">
+      <c r="M19" s="89" cm="1">
         <f t="array" ref="M19">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$7))</f>
         <v>519.2238834625033</v>
       </c>
-      <c r="N19" s="110" cm="1">
+      <c r="N19" s="109" cm="1">
         <f t="array" ref="N19">_xll.qlSwaptionAnnuity(L19,M19)</f>
         <v>56766.422970738087</v>
       </c>
@@ -7142,26 +7152,26 @@
         <f t="array" ref="Q19">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F19,S19,$C$22)</f>
         <v>6.8685932674608981E-3</v>
       </c>
-      <c r="R19" s="116">
-        <f>G19-F19</f>
+      <c r="R19" s="115">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="S19" s="117" t="str">
-        <f>ROUND(($C$17-G19)/365.25,0)&amp;"y"</f>
+      <c r="S19" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>7y</v>
       </c>
       <c r="T19" s="31" t="str" cm="1">
         <f t="array" ref="T19">_xll.qlSwaptionHelper(F19,S19,Q19,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R19,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C20SwaptionHelper,A</v>
       </c>
-      <c r="U19" s="69">
+      <c r="U19" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V19" s="118">
-        <f>$C$30</f>
+      <c r="V19" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W19" s="63" t="b" cm="1">
+      <c r="W19" s="62" t="b" cm="1">
         <f t="array" ref="W19">_xll.qlBlackCalibrationHelperSetPricingEngine(T19,$C$32)</f>
         <v>1</v>
       </c>
@@ -7169,8 +7179,8 @@
         <v>7.3317640293017773E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E20" s="98" t="s">
+    <row r="20" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E20" s="97" t="s">
         <v>104</v>
       </c>
       <c r="F20" s="32" cm="1">
@@ -7189,7 +7199,7 @@
         <f t="array" ref="I20">_xll.qlOvernightIndexedSwap("Payer",$C$21,H20,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J20" s="110" cm="1">
+      <c r="J20" s="109" cm="1">
         <f t="array" ref="J20">_xll.qlSwapLegBPS(I20,1,_xll.qlInstrumentSetPricingEngine(I20,$C$6))*10000</f>
         <v>47759.243446805121</v>
       </c>
@@ -7201,11 +7211,11 @@
         <f t="array" ref="L20">_xll.qlSwaption(I20,K20,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C12Swaption,A</v>
       </c>
-      <c r="M20" s="90" cm="1">
+      <c r="M20" s="89" cm="1">
         <f t="array" ref="M20">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$7))</f>
         <v>493.61995406800253</v>
       </c>
-      <c r="N20" s="110" cm="1">
+      <c r="N20" s="109" cm="1">
         <f t="array" ref="N20">_xll.qlSwaptionAnnuity(L20,M20)</f>
         <v>47759.243446805121</v>
       </c>
@@ -7217,26 +7227,26 @@
         <f t="array" ref="Q20">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F20,S20,$C$22)</f>
         <v>6.8710196098611381E-3</v>
       </c>
-      <c r="R20" s="116">
-        <f>G20-F20</f>
+      <c r="R20" s="115">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="S20" s="117" t="str">
-        <f>ROUND(($C$17-G20)/365.25,0)&amp;"y"</f>
+      <c r="S20" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>6y</v>
       </c>
       <c r="T20" s="31" t="str" cm="1">
         <f t="array" ref="T20">_xll.qlSwaptionHelper(F20,S20,Q20,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R20,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C20SwaptionHelper,A</v>
       </c>
-      <c r="U20" s="69">
+      <c r="U20" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V20" s="118">
-        <f>$C$30</f>
+      <c r="V20" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W20" s="63" t="b" cm="1">
+      <c r="W20" s="62" t="b" cm="1">
         <f t="array" ref="W20">_xll.qlBlackCalibrationHelperSetPricingEngine(T20,$C$32)</f>
         <v>1</v>
       </c>
@@ -7244,14 +7254,14 @@
         <v>7.2499818707807877E-3</v>
       </c>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B21" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="C21" s="82">
-        <v>10000</v>
-      </c>
-      <c r="E21" s="98" t="s">
+      <c r="C21" s="81">
+        <v>10000</v>
+      </c>
+      <c r="E21" s="97" t="s">
         <v>100</v>
       </c>
       <c r="F21" s="32" cm="1">
@@ -7270,7 +7280,7 @@
         <f t="array" ref="I21">_xll.qlOvernightIndexedSwap("Payer",$C$21,H21,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J21" s="110" cm="1">
+      <c r="J21" s="109" cm="1">
         <f t="array" ref="J21">_xll.qlSwapLegBPS(I21,1,_xll.qlInstrumentSetPricingEngine(I21,$C$6))*10000</f>
         <v>39055.847564585856</v>
       </c>
@@ -7282,11 +7292,11 @@
         <f t="array" ref="L21">_xll.qlSwaption(I21,K21,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C12Swaption,A</v>
       </c>
-      <c r="M21" s="90" cm="1">
+      <c r="M21" s="89" cm="1">
         <f t="array" ref="M21">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$7))</f>
         <v>445.14555434793988</v>
       </c>
-      <c r="N21" s="110" cm="1">
+      <c r="N21" s="109" cm="1">
         <f t="array" ref="N21">_xll.qlSwaptionAnnuity(L21,M21)</f>
         <v>39055.847564585856</v>
       </c>
@@ -7298,26 +7308,26 @@
         <f t="array" ref="Q21">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F21,S21,$C$22)</f>
         <v>6.8386420675278876E-3</v>
       </c>
-      <c r="R21" s="116">
-        <f>G21-F21</f>
+      <c r="R21" s="115">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="S21" s="117" t="str">
-        <f>ROUND(($C$17-G21)/365.25,0)&amp;"y"</f>
+      <c r="S21" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>5y</v>
       </c>
       <c r="T21" s="31" t="str" cm="1">
         <f t="array" ref="T21">_xll.qlSwaptionHelper(F21,S21,Q21,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R21,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C20SwaptionHelper,A</v>
       </c>
-      <c r="U21" s="69">
+      <c r="U21" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V21" s="118">
-        <f>$C$30</f>
+      <c r="V21" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W21" s="63" t="b" cm="1">
+      <c r="W21" s="62" t="b" cm="1">
         <f t="array" ref="W21">_xll.qlBlackCalibrationHelperSetPricingEngine(T21,$C$32)</f>
         <v>1</v>
       </c>
@@ -7325,14 +7335,14 @@
         <v>7.0519393916380711E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B22" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="C22" s="83">
+      <c r="C22" s="82">
         <v>0.03</v>
       </c>
-      <c r="E22" s="98" t="s">
+      <c r="E22" s="97" t="s">
         <v>105</v>
       </c>
       <c r="F22" s="32" cm="1">
@@ -7351,7 +7361,7 @@
         <f t="array" ref="I22">_xll.qlOvernightIndexedSwap("Payer",$C$21,H22,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J22" s="110" cm="1">
+      <c r="J22" s="109" cm="1">
         <f t="array" ref="J22">_xll.qlSwapLegBPS(I22,1,_xll.qlInstrumentSetPricingEngine(I22,$C$6))*10000</f>
         <v>30614.041334853744</v>
       </c>
@@ -7363,11 +7373,11 @@
         <f t="array" ref="L22">_xll.qlSwaption(I22,K22,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C12Swaption,A</v>
       </c>
-      <c r="M22" s="90" cm="1">
+      <c r="M22" s="89" cm="1">
         <f t="array" ref="M22">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$7))</f>
         <v>378.67641020372002</v>
       </c>
-      <c r="N22" s="110" cm="1">
+      <c r="N22" s="109" cm="1">
         <f t="array" ref="N22">_xll.qlSwaptionAnnuity(L22,M22)</f>
         <v>30614.04133485374</v>
       </c>
@@ -7379,26 +7389,26 @@
         <f t="array" ref="Q22">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F22,S22,$C$22)</f>
         <v>6.8094752901471274E-3</v>
       </c>
-      <c r="R22" s="116">
-        <f>G22-F22</f>
+      <c r="R22" s="115">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="S22" s="117" t="str">
-        <f>ROUND(($C$17-G22)/365.25,0)&amp;"y"</f>
+      <c r="S22" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>4y</v>
       </c>
       <c r="T22" s="31" t="str" cm="1">
         <f t="array" ref="T22">_xll.qlSwaptionHelper(F22,S22,Q22,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R22,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C20SwaptionHelper,A</v>
       </c>
-      <c r="U22" s="69">
+      <c r="U22" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V22" s="118">
-        <f>$C$30</f>
+      <c r="V22" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W22" s="63" t="b" cm="1">
+      <c r="W22" s="62" t="b" cm="1">
         <f t="array" ref="W22">_xll.qlBlackCalibrationHelperSetPricingEngine(T22,$C$32)</f>
         <v>1</v>
       </c>
@@ -7406,8 +7416,8 @@
         <v>7.0789799045768848E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E23" s="98" t="s">
+    <row r="23" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E23" s="97" t="s">
         <v>101</v>
       </c>
       <c r="F23" s="32" cm="1">
@@ -7426,7 +7436,7 @@
         <f t="array" ref="I23">_xll.qlOvernightIndexedSwap("Payer",$C$21,H23,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J23" s="110" cm="1">
+      <c r="J23" s="109" cm="1">
         <f t="array" ref="J23">_xll.qlSwapLegBPS(I23,1,_xll.qlInstrumentSetPricingEngine(I23,$C$6))*10000</f>
         <v>22505.50178121102</v>
       </c>
@@ -7438,11 +7448,11 @@
         <f t="array" ref="L23">_xll.qlSwaption(I23,K23,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C12Swaption,A</v>
       </c>
-      <c r="M23" s="90" cm="1">
+      <c r="M23" s="89" cm="1">
         <f t="array" ref="M23">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$7))</f>
         <v>298.39887641285605</v>
       </c>
-      <c r="N23" s="110" cm="1">
+      <c r="N23" s="109" cm="1">
         <f t="array" ref="N23">_xll.qlSwaptionAnnuity(L23,M23)</f>
         <v>22505.501781211016</v>
       </c>
@@ -7454,26 +7464,26 @@
         <f t="array" ref="Q23">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F23,S23,$C$22)</f>
         <v>6.7899775764584816E-3</v>
       </c>
-      <c r="R23" s="116">
-        <f>G23-F23</f>
+      <c r="R23" s="115">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="S23" s="117" t="str">
-        <f>ROUND(($C$17-G23)/365.25,0)&amp;"y"</f>
+      <c r="S23" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>3y</v>
       </c>
       <c r="T23" s="31" t="str" cm="1">
         <f t="array" ref="T23">_xll.qlSwaptionHelper(F23,S23,Q23,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R23,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C20SwaptionHelper,A</v>
       </c>
-      <c r="U23" s="69">
+      <c r="U23" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V23" s="118">
-        <f>$C$30</f>
+      <c r="V23" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W23" s="63" t="b" cm="1">
+      <c r="W23" s="62" t="b" cm="1">
         <f t="array" ref="W23">_xll.qlBlackCalibrationHelperSetPricingEngine(T23,$C$32)</f>
         <v>1</v>
       </c>
@@ -7481,8 +7491,8 @@
         <v>6.9660793842538805E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E24" s="98" t="s">
+    <row r="24" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E24" s="97" t="s">
         <v>106</v>
       </c>
       <c r="F24" s="32" cm="1">
@@ -7501,7 +7511,7 @@
         <f t="array" ref="I24">_xll.qlOvernightIndexedSwap("Payer",$C$21,H24,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J24" s="110" cm="1">
+      <c r="J24" s="109" cm="1">
         <f t="array" ref="J24">_xll.qlSwapLegBPS(I24,1,_xll.qlInstrumentSetPricingEngine(I24,$C$6))*10000</f>
         <v>14705.474136934443</v>
       </c>
@@ -7513,11 +7523,11 @@
         <f t="array" ref="L24">_xll.qlSwaption(I24,K24,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C12Swaption,A</v>
       </c>
-      <c r="M24" s="90" cm="1">
+      <c r="M24" s="89" cm="1">
         <f t="array" ref="M24">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$7))</f>
         <v>208.87169946565118</v>
       </c>
-      <c r="N24" s="110" cm="1">
+      <c r="N24" s="109" cm="1">
         <f t="array" ref="N24">_xll.qlSwaptionAnnuity(L24,M24)</f>
         <v>14705.474136934441</v>
       </c>
@@ -7529,26 +7539,26 @@
         <f t="array" ref="Q24">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F24,S24,$C$22)</f>
         <v>6.8705740176875649E-3</v>
       </c>
-      <c r="R24" s="116">
-        <f>G24-F24</f>
+      <c r="R24" s="115">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="S24" s="117" t="str">
-        <f>ROUND(($C$17-G24)/365.25,0)&amp;"y"</f>
+      <c r="S24" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>2y</v>
       </c>
       <c r="T24" s="31" t="str" cm="1">
         <f t="array" ref="T24">_xll.qlSwaptionHelper(F24,S24,Q24,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R24,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C20SwaptionHelper,A</v>
       </c>
-      <c r="U24" s="69">
+      <c r="U24" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V24" s="118">
-        <f>$C$30</f>
+      <c r="V24" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W24" s="63" t="b" cm="1">
+      <c r="W24" s="62" t="b" cm="1">
         <f t="array" ref="W24">_xll.qlBlackCalibrationHelperSetPricingEngine(T24,$C$32)</f>
         <v>1</v>
       </c>
@@ -7556,8 +7566,8 @@
         <v>7.8011054462023364E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="E25" s="99" t="s">
+    <row r="25" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="E25" s="98" t="s">
         <v>107</v>
       </c>
       <c r="F25" s="37" cm="1">
@@ -7576,7 +7586,7 @@
         <f t="array" ref="I25">_xll.qlOvernightIndexedSwap("Payer",$C$21,H25,$C$22,"Act/360",$C$19,0,0,"Following","TARGET")</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C9OvernightIndexedSwap,A</v>
       </c>
-      <c r="J25" s="111" cm="1">
+      <c r="J25" s="110" cm="1">
         <f t="array" ref="J25">_xll.qlSwapLegBPS(I25,1,_xll.qlInstrumentSetPricingEngine(I25,$C$6))*10000</f>
         <v>7171.0842364683413</v>
       </c>
@@ -7588,11 +7598,11 @@
         <f t="array" ref="L25">_xll.qlSwaption(I25,K25,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C12Swaption,A</v>
       </c>
-      <c r="M25" s="92" cm="1">
+      <c r="M25" s="91" cm="1">
         <f t="array" ref="M25">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$7))</f>
         <v>107.37919557367384</v>
       </c>
-      <c r="N25" s="111" cm="1">
+      <c r="N25" s="110" cm="1">
         <f t="array" ref="N25">_xll.qlSwaptionAnnuity(L25,M25)</f>
         <v>7171.0842364683413</v>
       </c>
@@ -7604,26 +7614,26 @@
         <f t="array" ref="Q25">_xll.qlSwaptionVolatilityStructureVolatility($C$5,F25,S25,$C$22)</f>
         <v>6.7898728295167242E-3</v>
       </c>
-      <c r="R25" s="116">
-        <f>G25-F25</f>
+      <c r="R25" s="115">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="S25" s="117" t="str">
-        <f>ROUND(($C$17-G25)/365.25,0)&amp;"y"</f>
+      <c r="S25" s="116" t="str">
+        <f t="shared" si="1"/>
         <v>1y</v>
       </c>
       <c r="T25" s="31" t="str" cm="1">
         <f t="array" ref="T25">_xll.qlSwaptionHelper(F25,S25,Q25,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R25,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C20SwaptionHelper,A</v>
       </c>
-      <c r="U25" s="69">
+      <c r="U25" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V25" s="118">
-        <f>$C$30</f>
+      <c r="V25" s="117">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
-      <c r="W25" s="63" t="b" cm="1">
+      <c r="W25" s="62" t="b" cm="1">
         <f t="array" ref="W25">_xll.qlBlackCalibrationHelperSetPricingEngine(T25,$C$32)</f>
         <v>1</v>
       </c>
@@ -7631,16 +7641,16 @@
         <v>6.4311298987523163E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:24" x14ac:dyDescent="0.3">
       <c r="Q26" s="34"/>
       <c r="R26" s="34"/>
       <c r="S26" s="34"/>
       <c r="T26" s="34"/>
-      <c r="U26" s="119">
+      <c r="U26" s="118">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="V26" s="120">
-        <f>$C$30</f>
+      <c r="V26" s="119">
+        <f t="shared" si="2"/>
         <v>0.01</v>
       </c>
       <c r="W26" s="39"/>
@@ -7648,47 +7658,47 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B30" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="C30" s="70">
+      <c r="C30" s="69">
         <v>0.01</v>
       </c>
     </row>
-    <row r="31" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>129</v>
       </c>
       <c r="C31" s="31" t="str" cm="1">
         <f t="array" ref="C31">_xll.qlGsr(C4,F17:F25,U17:U26,V17:V26,,M17:M25)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R31C3Gsr,B</v>
-      </c>
-    </row>
-    <row r="32" spans="2:24" x14ac:dyDescent="0.25">
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R31C3Gsr,A</v>
+      </c>
+    </row>
+    <row r="32" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>146</v>
       </c>
       <c r="C32" s="31" t="str" cm="1">
         <f t="array" ref="C32">_xll.qlGaussian1dJamshidianSwaptionEngine(C31)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R32C3Gaussian1dJamshidianSwaptionEngine,B</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R32C3Gaussian1dJamshidianSwaptionEngine,A</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33" s="34" t="s">
         <v>130</v>
       </c>
       <c r="C33" s="36" t="str" cm="1">
         <f t="array" ref="C33">_xll.qlGaussian1dSwaptionEngine(C31)</f>
-        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R33C3Gaussian1dSwaptionEngine,B</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+        <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R33C3Gaussian1dSwaptionEngine,A</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35" s="24" t="s">
         <v>134</v>
       </c>
@@ -7697,47 +7707,47 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R35C3LevenbergMarquardt,A</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="C36" s="84">
+      <c r="C36" s="83">
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="C37" s="84">
+      <c r="C37" s="83">
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>137</v>
       </c>
-      <c r="C38" s="85">
+      <c r="C38" s="84">
         <v>1E-4</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C39" s="85">
+      <c r="C39" s="84">
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="C40" s="85">
+      <c r="C40" s="84">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B41" s="34" t="s">
         <v>140</v>
       </c>
@@ -7746,21 +7756,21 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R41C3EndCriteria,A</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B43" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="C43" s="86" t="b" cm="1">
+      <c r="C43" s="85" t="b" cm="1">
         <f t="array" ref="C43">_xll.qlGsrCalibrateVolatilitiesIterative(C31,T17:T25,C35,C41,,,W17:W25)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B45" s="5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B47" s="24" t="s">
         <v>144</v>
       </c>
@@ -7769,7 +7779,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R47C3BermudanExercise,A</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B48" s="34" t="s">
         <v>143</v>
       </c>
@@ -7778,164 +7788,164 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R48C3Swaption,A</v>
       </c>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B50" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B52" s="22" t="s">
         <v>112</v>
       </c>
       <c r="C52" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="D52" s="93" t="s">
+      <c r="D52" s="92" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B53" s="87" t="str">
-        <f>E17&amp;"-"&amp;S17</f>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B53" s="86" t="str">
+        <f t="shared" ref="B53:B61" si="3">E17&amp;"-"&amp;S17</f>
         <v>1y-9y</v>
       </c>
-      <c r="C53" s="88" cm="1">
+      <c r="C53" s="87" cm="1">
         <f t="array" ref="C53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$32,$C$43))</f>
         <v>480.19295857890654</v>
       </c>
-      <c r="D53" s="88" cm="1">
+      <c r="D53" s="87" cm="1">
         <f t="array" ref="D53">_xll.qlInstrumentNPV(L17,_xll.qlInstrumentSetPricingEngine(L17,$C$33,$C$43))</f>
         <v>477.74924495888234</v>
       </c>
     </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B54" s="89" t="str">
-        <f>E18&amp;"-"&amp;S18</f>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B54" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>2y-8y</v>
       </c>
-      <c r="C54" s="90" cm="1">
+      <c r="C54" s="89" cm="1">
         <f t="array" ref="C54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$32,$C$43))</f>
         <v>514.75686806025317</v>
       </c>
-      <c r="D54" s="90" cm="1">
+      <c r="D54" s="89" cm="1">
         <f t="array" ref="D54">_xll.qlInstrumentNPV(L18,_xll.qlInstrumentSetPricingEngine(L18,$C$33,$C$43))</f>
         <v>513.50611040521835</v>
       </c>
     </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B55" s="89" t="str">
-        <f>E19&amp;"-"&amp;S19</f>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B55" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>3y-7y</v>
       </c>
-      <c r="C55" s="90" cm="1">
+      <c r="C55" s="89" cm="1">
         <f t="array" ref="C55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$32,$C$43))</f>
         <v>519.21992874969453</v>
       </c>
-      <c r="D55" s="90" cm="1">
+      <c r="D55" s="89" cm="1">
         <f t="array" ref="D55">_xll.qlInstrumentNPV(L19,_xll.qlInstrumentSetPricingEngine(L19,$C$33,$C$43))</f>
         <v>517.23545516948286</v>
       </c>
     </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B56" s="89" t="str">
-        <f>E20&amp;"-"&amp;S20</f>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B56" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>4y-6y</v>
       </c>
-      <c r="C56" s="90" cm="1">
+      <c r="C56" s="89" cm="1">
         <f t="array" ref="C56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$32,$C$43))</f>
         <v>493.60804779991349</v>
       </c>
-      <c r="D56" s="90" cm="1">
+      <c r="D56" s="89" cm="1">
         <f t="array" ref="D56">_xll.qlInstrumentNPV(L20,_xll.qlInstrumentSetPricingEngine(L20,$C$33,$C$43))</f>
         <v>491.03774318071919</v>
       </c>
     </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B57" s="89" t="str">
-        <f>E21&amp;"-"&amp;S21</f>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B57" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>5y-5y</v>
       </c>
-      <c r="C57" s="90" cm="1">
+      <c r="C57" s="89" cm="1">
         <f t="array" ref="C57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$32,$C$43))</f>
         <v>445.12383139248038</v>
       </c>
-      <c r="D57" s="90" cm="1">
+      <c r="D57" s="89" cm="1">
         <f t="array" ref="D57">_xll.qlInstrumentNPV(L21,_xll.qlInstrumentSetPricingEngine(L21,$C$33,$C$43))</f>
         <v>442.42184610809704</v>
       </c>
     </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B58" s="89" t="str">
-        <f>E22&amp;"-"&amp;S22</f>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B58" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>6y-4y</v>
       </c>
-      <c r="C58" s="90" cm="1">
+      <c r="C58" s="89" cm="1">
         <f t="array" ref="C58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$32,$C$43))</f>
         <v>378.66930593822264</v>
       </c>
-      <c r="D58" s="90" cm="1">
+      <c r="D58" s="89" cm="1">
         <f t="array" ref="D58">_xll.qlInstrumentNPV(L22,_xll.qlInstrumentSetPricingEngine(L22,$C$33,$C$43))</f>
         <v>376.09095103371908</v>
       </c>
     </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B59" s="89" t="str">
-        <f>E23&amp;"-"&amp;S23</f>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B59" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>7y-3y</v>
       </c>
-      <c r="C59" s="90" cm="1">
+      <c r="C59" s="89" cm="1">
         <f t="array" ref="C59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$32,$C$43))</f>
         <v>298.39373179886041</v>
       </c>
-      <c r="D59" s="90" cm="1">
+      <c r="D59" s="89" cm="1">
         <f t="array" ref="D59">_xll.qlInstrumentNPV(L23,_xll.qlInstrumentSetPricingEngine(L23,$C$33,$C$43))</f>
         <v>296.23172499493859</v>
       </c>
     </row>
-    <row r="60" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B60" s="89" t="str">
-        <f>E24&amp;"-"&amp;S24</f>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B60" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>8y-2y</v>
       </c>
-      <c r="C60" s="90" cm="1">
+      <c r="C60" s="89" cm="1">
         <f t="array" ref="C60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$32,$C$43))</f>
         <v>208.86665999869419</v>
       </c>
-      <c r="D60" s="90" cm="1">
+      <c r="D60" s="89" cm="1">
         <f t="array" ref="D60">_xll.qlInstrumentNPV(L24,_xll.qlInstrumentSetPricingEngine(L24,$C$33,$C$43))</f>
         <v>207.31794600871279</v>
       </c>
     </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B61" s="89" t="str">
-        <f>E25&amp;"-"&amp;S25</f>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B61" s="88" t="str">
+        <f t="shared" si="3"/>
         <v>9y-1y</v>
       </c>
-      <c r="C61" s="90" cm="1">
+      <c r="C61" s="89" cm="1">
         <f t="array" ref="C61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$32,$C$43))</f>
         <v>107.37144562488741</v>
       </c>
-      <c r="D61" s="90" cm="1">
+      <c r="D61" s="89" cm="1">
         <f t="array" ref="D61">_xll.qlInstrumentNPV(L25,_xll.qlInstrumentSetPricingEngine(L25,$C$33,$C$43))</f>
         <v>106.57878015619599</v>
       </c>
     </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B62" s="91" t="s">
+    <row r="62" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B62" s="90" t="s">
         <v>147</v>
       </c>
       <c r="C62" s="34"/>
-      <c r="D62" s="92" cm="1">
+      <c r="D62" s="91" cm="1">
         <f t="array" ref="D62">_xll.qlInstrumentNPV(C48,_xll.qlInstrumentSetPricingEngine(C48,$C$33,$C$43))</f>
         <v>631.27448041042044</v>
       </c>
     </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B64" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="C64" s="121"/>
-      <c r="D64" s="122">
+      <c r="C64" s="120"/>
+      <c r="D64" s="121">
         <f>D62-MAX(D53:D61)</f>
         <v>114.03902524093758</v>
       </c>

</xml_diff>